<commit_message>
Publish only the replicate rows in S1 and match its panel labels to Figure 6
The target-gene Ct sheet carried the lab workbook's closing summary block, in
Turkish, with group means and an interpretation column, and a per-replicate
column of direction notes. Neither is source data; both are dropped. In the
summary statistics the WST-1 rows are now panel 6C and the Fura-2 rows 6E,
as in Figure 6.
</commit_message>
<xml_diff>
--- a/supplementary/S1_laboratory_source_data.xlsx
+++ b/supplementary/S1_laboratory_source_data.xlsx
@@ -971,7 +971,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J65"/>
+  <dimension ref="A1:I57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1020,11 +1020,6 @@
           <t>rel_expression</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>note</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1060,7 +1055,6 @@
       <c r="I2" t="n">
         <v>1.022782938747284</v>
       </c>
-      <c r="J2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1096,7 +1090,6 @@
       <c r="I3" t="n">
         <v>0.967611620142344</v>
       </c>
-      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1132,7 +1125,6 @@
       <c r="I4" t="n">
         <v>1.008701983790398</v>
       </c>
-      <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1168,7 +1160,6 @@
       <c r="I5" t="n">
         <v>1.001734370234696</v>
       </c>
-      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1204,11 +1195,6 @@
       <c r="I6" t="n">
         <v>1.818186259055118</v>
       </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1244,11 +1230,6 @@
       <c r="I7" t="n">
         <v>1.518345380207591</v>
       </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1284,11 +1265,6 @@
       <c r="I8" t="n">
         <v>1.90858045006437</v>
       </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1324,11 +1300,6 @@
       <c r="I9" t="n">
         <v>2.031436121861929</v>
       </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1364,7 +1335,6 @@
       <c r="I10" t="n">
         <v>1.033472499899176</v>
       </c>
-      <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1400,7 +1370,6 @@
       <c r="I11" t="n">
         <v>1.04789923837507</v>
       </c>
-      <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1436,7 +1405,6 @@
       <c r="I12" t="n">
         <v>1.055187953981984</v>
       </c>
-      <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1472,7 +1440,6 @@
       <c r="I13" t="n">
         <v>0.8750879947452087</v>
       </c>
-      <c r="J13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1508,11 +1475,6 @@
       <c r="I14" t="n">
         <v>1.714157888456202</v>
       </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1548,11 +1510,6 @@
       <c r="I15" t="n">
         <v>1.471716715625615</v>
       </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1588,11 +1545,6 @@
       <c r="I16" t="n">
         <v>1.566451389130095</v>
       </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1628,11 +1580,6 @@
       <c r="I17" t="n">
         <v>1.969050346674829</v>
       </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1668,7 +1615,6 @@
       <c r="I18" t="n">
         <v>1.154685531688693</v>
       </c>
-      <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1704,7 +1650,6 @@
       <c r="I19" t="n">
         <v>0.9913730874626632</v>
       </c>
-      <c r="J19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1740,7 +1685,6 @@
       <c r="I20" t="n">
         <v>1.005212140041474</v>
       </c>
-      <c r="J20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1776,7 +1720,6 @@
       <c r="I21" t="n">
         <v>0.8690433204285118</v>
       </c>
-      <c r="J21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1812,11 +1755,6 @@
       <c r="I22" t="n">
         <v>2.862945089285228</v>
       </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1852,11 +1790,6 @@
       <c r="I23" t="n">
         <v>2.963906629820919</v>
       </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1892,11 +1825,6 @@
       <c r="I24" t="n">
         <v>3.883883697369405</v>
       </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1932,11 +1860,6 @@
       <c r="I25" t="n">
         <v>3.089771179918305</v>
       </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1972,7 +1895,6 @@
       <c r="I26" t="n">
         <v>0.9913730874626625</v>
       </c>
-      <c r="J26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2008,7 +1930,6 @@
       <c r="I27" t="n">
         <v>1.033472499899175</v>
       </c>
-      <c r="J27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2044,7 +1965,6 @@
       <c r="I28" t="n">
         <v>0.9982686325973916</v>
       </c>
-      <c r="J28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2080,7 +2000,6 @@
       <c r="I29" t="n">
         <v>0.9777245612102334</v>
       </c>
-      <c r="J29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2116,11 +2035,6 @@
       <c r="I30" t="n">
         <v>1.941941848684702</v>
       </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2156,11 +2070,6 @@
       <c r="I31" t="n">
         <v>1.49226111537404</v>
       </c>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2196,11 +2105,6 @@
       <c r="I32" t="n">
         <v>1.655767377972946</v>
       </c>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2236,11 +2140,6 @@
       <c r="I33" t="n">
         <v>1.824498544489991</v>
       </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2276,7 +2175,6 @@
       <c r="I34" t="n">
         <v>1.051537280994008</v>
       </c>
-      <c r="J34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2312,7 +2210,6 @@
       <c r="I35" t="n">
         <v>0.8965773757702972</v>
       </c>
-      <c r="J35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2348,7 +2245,6 @@
       <c r="I36" t="n">
         <v>1.066216194416503</v>
       </c>
-      <c r="J36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2384,7 +2280,6 @@
       <c r="I37" t="n">
         <v>0.9948148855014215</v>
       </c>
-      <c r="J37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2420,11 +2315,6 @@
       <c r="I38" t="n">
         <v>0.5008671851173484</v>
       </c>
-      <c r="J38" t="inlineStr">
-        <is>
-          <t>DOWN (sig)</t>
-        </is>
-      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2460,11 +2350,6 @@
       <c r="I39" t="n">
         <v>0.5149484783374492</v>
       </c>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>DOWN (sig)</t>
-        </is>
-      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2500,11 +2385,6 @@
       <c r="I40" t="n">
         <v>0.4974074427507107</v>
       </c>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t>DOWN (sig)</t>
-        </is>
-      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2540,11 +2420,6 @@
       <c r="I41" t="n">
         <v>0.5043509918951993</v>
       </c>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>DOWN (sig)</t>
-        </is>
-      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2580,7 +2455,6 @@
       <c r="I42" t="n">
         <v>0.9090931295275597</v>
       </c>
-      <c r="J42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2616,7 +2490,6 @@
       <c r="I43" t="n">
         <v>1.191269640425871</v>
       </c>
-      <c r="J43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2652,7 +2525,6 @@
       <c r="I44" t="n">
         <v>0.7914115359988518</v>
       </c>
-      <c r="J44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2688,7 +2560,6 @@
       <c r="I45" t="n">
         <v>1.166753665732178</v>
       </c>
-      <c r="J45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2724,11 +2595,6 @@
       <c r="I46" t="n">
         <v>0.8307578929497527</v>
       </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>DOWN (ns)</t>
-        </is>
-      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2764,11 +2630,6 @@
       <c r="I47" t="n">
         <v>0.7435491420613253</v>
       </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>DOWN (ns)</t>
-        </is>
-      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2804,11 +2665,6 @@
       <c r="I48" t="n">
         <v>0.9542902250321834</v>
       </c>
-      <c r="J48" t="inlineStr">
-        <is>
-          <t>DOWN (ns)</t>
-        </is>
-      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2844,11 +2700,6 @@
       <c r="I49" t="n">
         <v>0.8307578929497527</v>
       </c>
-      <c r="J49" t="inlineStr">
-        <is>
-          <t>DOWN (ns)</t>
-        </is>
-      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2884,7 +2735,6 @@
       <c r="I50" t="n">
         <v>1.012203943399157</v>
       </c>
-      <c r="J50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2920,7 +2770,6 @@
       <c r="I51" t="n">
         <v>0.9576032806985754</v>
       </c>
-      <c r="J51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2956,7 +2805,6 @@
       <c r="I52" t="n">
         <v>1.026333783890422</v>
       </c>
-      <c r="J52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2992,7 +2840,6 @@
       <c r="I53" t="n">
         <v>1.005212140041476</v>
       </c>
-      <c r="J53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3028,11 +2875,6 @@
       <c r="I54" t="n">
         <v>1.901977263335279</v>
       </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3068,11 +2910,6 @@
       <c r="I55" t="n">
         <v>1.523616693518236</v>
       </c>
-      <c r="J55" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3108,11 +2945,6 @@
       <c r="I56" t="n">
         <v>1.955449122420466</v>
       </c>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3148,271 +2980,6 @@
       <c r="I57" t="n">
         <v>2.154719391831541</v>
       </c>
-      <c r="J57" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>Gene</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>Kontrol mean</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>shTDP-43 mean</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>Yön</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>Anlamlılık (beklenen)</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>Not</t>
-        </is>
-      </c>
-      <c r="G58" t="inlineStr"/>
-      <c r="H58" t="inlineStr"/>
-      <c r="I58" t="inlineStr"/>
-      <c r="J58" t="inlineStr"/>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>TRPC1</t>
-        </is>
-      </c>
-      <c r="B59" t="n">
-        <v>1.000207728228681</v>
-      </c>
-      <c r="C59" t="n">
-        <v>1.819137052797252</v>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>Anlamlı artış</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>SOCE bileşeni</t>
-        </is>
-      </c>
-      <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr"/>
-      <c r="I59" t="inlineStr"/>
-      <c r="J59" t="inlineStr"/>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>ORAI1</t>
-        </is>
-      </c>
-      <c r="B60" t="n">
-        <v>1.002911921750359</v>
-      </c>
-      <c r="C60" t="n">
-        <v>1.680344084971685</v>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>Anlamlı artış</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>SOCE bileşeni</t>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr"/>
-      <c r="I60" t="inlineStr"/>
-      <c r="J60" t="inlineStr"/>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>ATP2A3</t>
-        </is>
-      </c>
-      <c r="B61" t="n">
-        <v>1.005078519905336</v>
-      </c>
-      <c r="C61" t="n">
-        <v>3.200126649098464</v>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>Anlamlı artış</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>SERCA3 – ER Ca²⁺</t>
-        </is>
-      </c>
-      <c r="G61" t="inlineStr"/>
-      <c r="H61" t="inlineStr"/>
-      <c r="I61" t="inlineStr"/>
-      <c r="J61" t="inlineStr"/>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>BCL2</t>
-        </is>
-      </c>
-      <c r="B62" t="n">
-        <v>1.000209695292366</v>
-      </c>
-      <c r="C62" t="n">
-        <v>1.72861722163042</v>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>Anlamlı artış</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>Anti-apoptotik</t>
-        </is>
-      </c>
-      <c r="G62" t="inlineStr"/>
-      <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr"/>
-      <c r="J62" t="inlineStr"/>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>BAK1</t>
-        </is>
-      </c>
-      <c r="B63" t="n">
-        <v>1.002286434170557</v>
-      </c>
-      <c r="C63" t="n">
-        <v>0.5043935245251769</v>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>Anlamlı azalma</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>Pro-apoptotik</t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr"/>
-      <c r="H63" t="inlineStr"/>
-      <c r="I63" t="inlineStr"/>
-      <c r="J63" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>BAX</t>
-        </is>
-      </c>
-      <c r="B64" t="n">
-        <v>1.014631992921115</v>
-      </c>
-      <c r="C64" t="n">
-        <v>0.8398387882482534</v>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>Azalma (anlamsız)</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>Pro-apoptotik</t>
-        </is>
-      </c>
-      <c r="G64" t="inlineStr"/>
-      <c r="H64" t="inlineStr"/>
-      <c r="I64" t="inlineStr"/>
-      <c r="J64" t="inlineStr"/>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>STIM1</t>
-        </is>
-      </c>
-      <c r="B65" t="n">
-        <v>1.000338287007407</v>
-      </c>
-      <c r="C65" t="n">
-        <v>1.88394061777638</v>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>UP</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>Anlamlı artış</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>SOCE – ER Ca²⁺ sensor</t>
-        </is>
-      </c>
-      <c r="G65" t="inlineStr"/>
-      <c r="H65" t="inlineStr"/>
-      <c r="I65" t="inlineStr"/>
-      <c r="J65" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5472,7 +5039,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ER Ca2+ release delta F340/F380</t>
+          <t>WST-1 viability 24 h</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -5481,13 +5048,13 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E14" t="n">
-        <v>0.268</v>
+        <v>100</v>
       </c>
       <c r="F14" t="n">
-        <v>0.042</v>
+        <v>1.5</v>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
@@ -5500,7 +5067,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ER Ca2+ release delta F340/F380</t>
+          <t>WST-1 viability 24 h</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -5509,13 +5076,13 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E15" t="n">
-        <v>0.18</v>
+        <v>116.8</v>
       </c>
       <c r="F15" t="n">
-        <v>0.061</v>
+        <v>1.6</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -5524,7 +5091,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>0.2989</t>
+          <t>0.000243</t>
         </is>
       </c>
     </row>
@@ -5536,7 +5103,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>SOCE delta F340/F380</t>
+          <t>WST-1 viability 48 h</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -5545,13 +5112,13 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E16" t="n">
-        <v>1.542</v>
+        <v>100</v>
       </c>
       <c r="F16" t="n">
-        <v>0.282</v>
+        <v>1.2</v>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
@@ -5564,7 +5131,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>SOCE delta F340/F380</t>
+          <t>WST-1 viability 48 h</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -5573,13 +5140,13 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E17" t="n">
-        <v>0.245</v>
+        <v>61.5</v>
       </c>
       <c r="F17" t="n">
-        <v>0.083</v>
+        <v>0.8</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -5588,19 +5155,19 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>0.0115</t>
+          <t>2.14e-07</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>6D</t>
+          <t>6E</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>WST-1 viability 24 h</t>
+          <t>ER Ca2+ release delta F340/F380</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -5609,13 +5176,13 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E18" t="n">
-        <v>100</v>
+        <v>0.268</v>
       </c>
       <c r="F18" t="n">
-        <v>1.5</v>
+        <v>0.042</v>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
@@ -5623,12 +5190,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>6D</t>
+          <t>6E</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>WST-1 viability 24 h</t>
+          <t>ER Ca2+ release delta F340/F380</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -5637,13 +5204,13 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E19" t="n">
-        <v>116.8</v>
+        <v>0.18</v>
       </c>
       <c r="F19" t="n">
-        <v>1.6</v>
+        <v>0.061</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -5652,19 +5219,19 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>0.000243</t>
+          <t>0.2989</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>6D</t>
+          <t>6E</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>WST-1 viability 48 h</t>
+          <t>SOCE delta F340/F380</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -5673,13 +5240,13 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E20" t="n">
-        <v>100</v>
+        <v>1.542</v>
       </c>
       <c r="F20" t="n">
-        <v>1.2</v>
+        <v>0.282</v>
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
@@ -5687,12 +5254,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>6D</t>
+          <t>6E</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>WST-1 viability 48 h</t>
+          <t>SOCE delta F340/F380</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -5701,13 +5268,13 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E21" t="n">
-        <v>61.5</v>
+        <v>0.245</v>
       </c>
       <c r="F21" t="n">
-        <v>0.8</v>
+        <v>0.083</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -5716,7 +5283,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2.14e-07</t>
+          <t>0.0115</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Name the laboratory control group, drop the apoptosis markers, remove revision wording
- The target-gene RT-qPCR, Fura-2 and WST-1 experiments compare shTDP-43
  cells with the non-targeting (scrambled) shRNA control; Methods 2.12-2.15,
  Section 3.7, the Figure 6 legend and labels, S1 and the graphical abstract
  now say so. For TARDBP the calibrator is the non-transduced group.
- S1 keeps the four targets reported in the manuscript; the apoptosis
  markers measured on the same RNA are not part of this study.
- Wording that referred to earlier versions ("before the correction",
  "no longer", "our first attempt", "the corrected analysis" and similar)
  is rewritten as method description; the effect of counting reference
  skips (+0.489 instead of +0.145) is kept as a sensitivity note in
  Methods 2.7, and the gene-level STMN2 sentence now reports the current
  eleven regions. The consistency check forbids the old phrases (275 checks).
</commit_message>
<xml_diff>
--- a/supplementary/S1_laboratory_source_data.xlsx
+++ b/supplementary/S1_laboratory_source_data.xlsx
@@ -468,7 +468,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Raw Ct values for the SOCE and apoptosis targets, four biological replicates per group, same RNA set; experiment window 03.06-10.07.2026.</t>
+          <t>Raw Ct values for the four SOCE-associated targets and GAPDH in shTDP-43 cells and the non-targeting (scrambled) shRNA control, four biological replicates per group, same RNA set; experiment window 03.06-10.07.2026.</t>
         </is>
       </c>
     </row>
@@ -492,7 +492,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Fura-2/AM measurements. ER Ca2+ release is the rise in F340/F380 after 10 uM cyclopiazonic acid in Ca2+-free HBS with EGTA; SOCE is the rise after re-addition of 1.5 mM CaCl2. Both as delta(F340/F380) versus the preceding baseline. The three samples of each group come from three independent cultures.</t>
+          <t>Fura-2/AM measurements. ER Ca2+ release is the rise in F340/F380 after 10 uM cyclopiazonic acid in Ca2+-free HBS with EGTA; SOCE is the rise after re-addition of 1.5 mM CaCl2. Both as delta(F340/F380) versus the preceding baseline. The three samples of each group come from three independent cultures. The control group is the non-targeting (scrambled) shRNA control.</t>
         </is>
       </c>
     </row>
@@ -504,7 +504,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>WST-1 viability, four wells per group, normalised to the mean of the control group at the same time point.</t>
+          <t>WST-1 viability, four wells per group, normalised to the mean of the non-targeting (scrambled) shRNA control at the same time point.</t>
         </is>
       </c>
     </row>
@@ -971,7 +971,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I57"/>
+  <dimension ref="A1:I33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1029,7 +1029,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -1064,7 +1064,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -1099,7 +1099,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1134,7 +1134,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1309,7 +1309,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1344,7 +1344,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1379,7 +1379,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1414,7 +1414,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -1589,7 +1589,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -1624,7 +1624,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -1659,7 +1659,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -1694,7 +1694,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -1864,12 +1864,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>BCL2</t>
+          <t>STIM1</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -1881,30 +1881,30 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>24.93</v>
+        <v>25.64</v>
       </c>
       <c r="F26" t="n">
         <v>19.42</v>
       </c>
       <c r="G26" t="n">
-        <v>5.509999999999998</v>
+        <v>6.219999999999999</v>
       </c>
       <c r="H26" t="n">
-        <v>0.01249999999999929</v>
+        <v>-0.01750000000000096</v>
       </c>
       <c r="I26" t="n">
-        <v>0.9913730874626625</v>
+        <v>1.012203943399157</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>BCL2</t>
+          <t>STIM1</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -1916,30 +1916,30 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>25.12</v>
+        <v>25.97</v>
       </c>
       <c r="F27" t="n">
         <v>19.67</v>
       </c>
       <c r="G27" t="n">
-        <v>5.449999999999999</v>
+        <v>6.299999999999997</v>
       </c>
       <c r="H27" t="n">
-        <v>-0.04749999999999943</v>
+        <v>0.06249999999999734</v>
       </c>
       <c r="I27" t="n">
-        <v>1.033472499899175</v>
+        <v>0.9576032806985754</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>BCL2</t>
+          <t>STIM1</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -1951,30 +1951,30 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>24.81</v>
+        <v>25.51</v>
       </c>
       <c r="F28" t="n">
         <v>19.31</v>
       </c>
       <c r="G28" t="n">
-        <v>5.5</v>
+        <v>6.200000000000003</v>
       </c>
       <c r="H28" t="n">
-        <v>0.002500000000001279</v>
+        <v>-0.03749999999999698</v>
       </c>
       <c r="I28" t="n">
-        <v>0.9982686325973916</v>
+        <v>1.026333783890422</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>BCL2</t>
+          <t>STIM1</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -1986,25 +1986,25 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>25.08</v>
+        <v>25.78</v>
       </c>
       <c r="F29" t="n">
         <v>19.55</v>
       </c>
       <c r="G29" t="n">
-        <v>5.529999999999998</v>
+        <v>6.23</v>
       </c>
       <c r="H29" t="n">
-        <v>0.03249999999999886</v>
+        <v>-0.007499999999999396</v>
       </c>
       <c r="I29" t="n">
-        <v>0.9777245612102334</v>
+        <v>1.005212140041476</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>BCL2</t>
+          <t>STIM1</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2021,25 +2021,25 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>24.02</v>
+        <v>24.79</v>
       </c>
       <c r="F30" t="n">
         <v>19.48</v>
       </c>
       <c r="G30" t="n">
-        <v>4.539999999999999</v>
+        <v>5.309999999999999</v>
       </c>
       <c r="H30" t="n">
-        <v>-0.9574999999999996</v>
+        <v>-0.9275000000000011</v>
       </c>
       <c r="I30" t="n">
-        <v>1.941941848684702</v>
+        <v>1.901977263335279</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>BCL2</t>
+          <t>STIM1</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2056,25 +2056,25 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>24.31</v>
+        <v>25.02</v>
       </c>
       <c r="F31" t="n">
         <v>19.39</v>
       </c>
       <c r="G31" t="n">
-        <v>4.919999999999998</v>
+        <v>5.629999999999999</v>
       </c>
       <c r="H31" t="n">
-        <v>-0.5775000000000006</v>
+        <v>-0.6075000000000008</v>
       </c>
       <c r="I31" t="n">
-        <v>1.49226111537404</v>
+        <v>1.523616693518236</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>BCL2</t>
+          <t>STIM1</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2091,25 +2091,25 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>24.38</v>
+        <v>24.88</v>
       </c>
       <c r="F32" t="n">
         <v>19.61</v>
       </c>
       <c r="G32" t="n">
-        <v>4.77</v>
+        <v>5.27</v>
       </c>
       <c r="H32" t="n">
-        <v>-0.7274999999999991</v>
+        <v>-0.9675000000000002</v>
       </c>
       <c r="I32" t="n">
-        <v>1.655767377972946</v>
+        <v>1.955449122420466</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>BCL2</t>
+          <t>STIM1</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2126,858 +2126,18 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>24.15</v>
+        <v>24.65</v>
       </c>
       <c r="F33" t="n">
         <v>19.52</v>
       </c>
       <c r="G33" t="n">
-        <v>4.629999999999999</v>
+        <v>5.129999999999999</v>
       </c>
       <c r="H33" t="n">
-        <v>-0.8674999999999997</v>
+        <v>-1.107500000000001</v>
       </c>
       <c r="I33" t="n">
-        <v>1.824498544489991</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>BAK1</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Control</t>
-        </is>
-      </c>
-      <c r="C34" t="n">
-        <v>1</v>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>03.06.2026</t>
-        </is>
-      </c>
-      <c r="E34" t="n">
-        <v>25.41</v>
-      </c>
-      <c r="F34" t="n">
-        <v>19.42</v>
-      </c>
-      <c r="G34" t="n">
-        <v>5.989999999999998</v>
-      </c>
-      <c r="H34" t="n">
-        <v>-0.07250000000000156</v>
-      </c>
-      <c r="I34" t="n">
-        <v>1.051537280994008</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>BAK1</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Control</t>
-        </is>
-      </c>
-      <c r="C35" t="n">
-        <v>2</v>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>11.06.2026</t>
-        </is>
-      </c>
-      <c r="E35" t="n">
-        <v>25.89</v>
-      </c>
-      <c r="F35" t="n">
-        <v>19.67</v>
-      </c>
-      <c r="G35" t="n">
-        <v>6.219999999999999</v>
-      </c>
-      <c r="H35" t="n">
-        <v>0.1574999999999989</v>
-      </c>
-      <c r="I35" t="n">
-        <v>0.8965773757702972</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>BAK1</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Control</t>
-        </is>
-      </c>
-      <c r="C36" t="n">
-        <v>3</v>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>25.06.2026</t>
-        </is>
-      </c>
-      <c r="E36" t="n">
-        <v>25.28</v>
-      </c>
-      <c r="F36" t="n">
-        <v>19.31</v>
-      </c>
-      <c r="G36" t="n">
-        <v>5.970000000000002</v>
-      </c>
-      <c r="H36" t="n">
-        <v>-0.09249999999999758</v>
-      </c>
-      <c r="I36" t="n">
-        <v>1.066216194416503</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>BAK1</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Control</t>
-        </is>
-      </c>
-      <c r="C37" t="n">
-        <v>4</v>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>09.07.2026</t>
-        </is>
-      </c>
-      <c r="E37" t="n">
-        <v>25.62</v>
-      </c>
-      <c r="F37" t="n">
-        <v>19.55</v>
-      </c>
-      <c r="G37" t="n">
-        <v>6.07</v>
-      </c>
-      <c r="H37" t="n">
-        <v>0.007500000000000284</v>
-      </c>
-      <c r="I37" t="n">
-        <v>0.9948148855014215</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>BAK1</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>shTDP-43</t>
-        </is>
-      </c>
-      <c r="C38" t="n">
-        <v>1</v>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>04.06.2026</t>
-        </is>
-      </c>
-      <c r="E38" t="n">
-        <v>26.54</v>
-      </c>
-      <c r="F38" t="n">
-        <v>19.48</v>
-      </c>
-      <c r="G38" t="n">
-        <v>7.059999999999999</v>
-      </c>
-      <c r="H38" t="n">
-        <v>0.9974999999999987</v>
-      </c>
-      <c r="I38" t="n">
-        <v>0.5008671851173484</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>BAK1</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>shTDP-43</t>
-        </is>
-      </c>
-      <c r="C39" t="n">
-        <v>2</v>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>12.06.2026</t>
-        </is>
-      </c>
-      <c r="E39" t="n">
-        <v>26.41</v>
-      </c>
-      <c r="F39" t="n">
-        <v>19.39</v>
-      </c>
-      <c r="G39" t="n">
-        <v>7.02</v>
-      </c>
-      <c r="H39" t="n">
-        <v>0.9574999999999996</v>
-      </c>
-      <c r="I39" t="n">
-        <v>0.5149484783374492</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>BAK1</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>shTDP-43</t>
-        </is>
-      </c>
-      <c r="C40" t="n">
-        <v>3</v>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>26.06.2026</t>
-        </is>
-      </c>
-      <c r="E40" t="n">
-        <v>26.68</v>
-      </c>
-      <c r="F40" t="n">
-        <v>19.61</v>
-      </c>
-      <c r="G40" t="n">
-        <v>7.07</v>
-      </c>
-      <c r="H40" t="n">
-        <v>1.0075</v>
-      </c>
-      <c r="I40" t="n">
-        <v>0.4974074427507107</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>BAK1</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>shTDP-43</t>
-        </is>
-      </c>
-      <c r="C41" t="n">
-        <v>4</v>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>10.07.2026</t>
-        </is>
-      </c>
-      <c r="E41" t="n">
-        <v>26.57</v>
-      </c>
-      <c r="F41" t="n">
-        <v>19.52</v>
-      </c>
-      <c r="G41" t="n">
-        <v>7.050000000000001</v>
-      </c>
-      <c r="H41" t="n">
-        <v>0.9875000000000007</v>
-      </c>
-      <c r="I41" t="n">
-        <v>0.5043509918951993</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>BAX</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Control</t>
-        </is>
-      </c>
-      <c r="C42" t="n">
-        <v>1</v>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>03.06.2026</t>
-        </is>
-      </c>
-      <c r="E42" t="n">
-        <v>26.72</v>
-      </c>
-      <c r="F42" t="n">
-        <v>19.42</v>
-      </c>
-      <c r="G42" t="n">
-        <v>7.299999999999997</v>
-      </c>
-      <c r="H42" t="n">
-        <v>0.1374999999999993</v>
-      </c>
-      <c r="I42" t="n">
-        <v>0.9090931295275597</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>BAX</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Control</t>
-        </is>
-      </c>
-      <c r="C43" t="n">
-        <v>2</v>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>11.06.2026</t>
-        </is>
-      </c>
-      <c r="E43" t="n">
-        <v>26.58</v>
-      </c>
-      <c r="F43" t="n">
-        <v>19.67</v>
-      </c>
-      <c r="G43" t="n">
-        <v>6.909999999999997</v>
-      </c>
-      <c r="H43" t="n">
-        <v>-0.2525000000000013</v>
-      </c>
-      <c r="I43" t="n">
-        <v>1.191269640425871</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>BAX</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Control</t>
-        </is>
-      </c>
-      <c r="C44" t="n">
-        <v>3</v>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>25.06.2026</t>
-        </is>
-      </c>
-      <c r="E44" t="n">
-        <v>26.81</v>
-      </c>
-      <c r="F44" t="n">
-        <v>19.31</v>
-      </c>
-      <c r="G44" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="H44" t="n">
-        <v>0.3375000000000021</v>
-      </c>
-      <c r="I44" t="n">
-        <v>0.7914115359988518</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>BAX</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Control</t>
-        </is>
-      </c>
-      <c r="C45" t="n">
-        <v>4</v>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>09.07.2026</t>
-        </is>
-      </c>
-      <c r="E45" t="n">
-        <v>26.49</v>
-      </c>
-      <c r="F45" t="n">
-        <v>19.55</v>
-      </c>
-      <c r="G45" t="n">
-        <v>6.939999999999998</v>
-      </c>
-      <c r="H45" t="n">
-        <v>-0.2225000000000001</v>
-      </c>
-      <c r="I45" t="n">
-        <v>1.166753665732178</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>BAX</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>shTDP-43</t>
-        </is>
-      </c>
-      <c r="C46" t="n">
-        <v>1</v>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>04.06.2026</t>
-        </is>
-      </c>
-      <c r="E46" t="n">
-        <v>26.91</v>
-      </c>
-      <c r="F46" t="n">
-        <v>19.48</v>
-      </c>
-      <c r="G46" t="n">
-        <v>7.43</v>
-      </c>
-      <c r="H46" t="n">
-        <v>0.2675000000000018</v>
-      </c>
-      <c r="I46" t="n">
-        <v>0.8307578929497527</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>BAX</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>shTDP-43</t>
-        </is>
-      </c>
-      <c r="C47" t="n">
-        <v>2</v>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>12.06.2026</t>
-        </is>
-      </c>
-      <c r="E47" t="n">
-        <v>26.98</v>
-      </c>
-      <c r="F47" t="n">
-        <v>19.39</v>
-      </c>
-      <c r="G47" t="n">
-        <v>7.59</v>
-      </c>
-      <c r="H47" t="n">
-        <v>0.427500000000002</v>
-      </c>
-      <c r="I47" t="n">
-        <v>0.7435491420613253</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>BAX</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>shTDP-43</t>
-        </is>
-      </c>
-      <c r="C48" t="n">
-        <v>3</v>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>26.06.2026</t>
-        </is>
-      </c>
-      <c r="E48" t="n">
-        <v>26.84</v>
-      </c>
-      <c r="F48" t="n">
-        <v>19.61</v>
-      </c>
-      <c r="G48" t="n">
-        <v>7.23</v>
-      </c>
-      <c r="H48" t="n">
-        <v>0.06750000000000256</v>
-      </c>
-      <c r="I48" t="n">
-        <v>0.9542902250321834</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>BAX</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>shTDP-43</t>
-        </is>
-      </c>
-      <c r="C49" t="n">
-        <v>4</v>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>10.07.2026</t>
-        </is>
-      </c>
-      <c r="E49" t="n">
-        <v>26.95</v>
-      </c>
-      <c r="F49" t="n">
-        <v>19.52</v>
-      </c>
-      <c r="G49" t="n">
-        <v>7.43</v>
-      </c>
-      <c r="H49" t="n">
-        <v>0.2675000000000018</v>
-      </c>
-      <c r="I49" t="n">
-        <v>0.8307578929497527</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>STIM1</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>Control</t>
-        </is>
-      </c>
-      <c r="C50" t="n">
-        <v>1</v>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>03.06.2026</t>
-        </is>
-      </c>
-      <c r="E50" t="n">
-        <v>25.64</v>
-      </c>
-      <c r="F50" t="n">
-        <v>19.42</v>
-      </c>
-      <c r="G50" t="n">
-        <v>6.219999999999999</v>
-      </c>
-      <c r="H50" t="n">
-        <v>-0.01750000000000096</v>
-      </c>
-      <c r="I50" t="n">
-        <v>1.012203943399157</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>STIM1</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>Control</t>
-        </is>
-      </c>
-      <c r="C51" t="n">
-        <v>2</v>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>11.06.2026</t>
-        </is>
-      </c>
-      <c r="E51" t="n">
-        <v>25.97</v>
-      </c>
-      <c r="F51" t="n">
-        <v>19.67</v>
-      </c>
-      <c r="G51" t="n">
-        <v>6.299999999999997</v>
-      </c>
-      <c r="H51" t="n">
-        <v>0.06249999999999734</v>
-      </c>
-      <c r="I51" t="n">
-        <v>0.9576032806985754</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>STIM1</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>Control</t>
-        </is>
-      </c>
-      <c r="C52" t="n">
-        <v>3</v>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>25.06.2026</t>
-        </is>
-      </c>
-      <c r="E52" t="n">
-        <v>25.51</v>
-      </c>
-      <c r="F52" t="n">
-        <v>19.31</v>
-      </c>
-      <c r="G52" t="n">
-        <v>6.200000000000003</v>
-      </c>
-      <c r="H52" t="n">
-        <v>-0.03749999999999698</v>
-      </c>
-      <c r="I52" t="n">
-        <v>1.026333783890422</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>STIM1</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>Control</t>
-        </is>
-      </c>
-      <c r="C53" t="n">
-        <v>4</v>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>09.07.2026</t>
-        </is>
-      </c>
-      <c r="E53" t="n">
-        <v>25.78</v>
-      </c>
-      <c r="F53" t="n">
-        <v>19.55</v>
-      </c>
-      <c r="G53" t="n">
-        <v>6.23</v>
-      </c>
-      <c r="H53" t="n">
-        <v>-0.007499999999999396</v>
-      </c>
-      <c r="I53" t="n">
-        <v>1.005212140041476</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>STIM1</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>shTDP-43</t>
-        </is>
-      </c>
-      <c r="C54" t="n">
-        <v>1</v>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>04.06.2026</t>
-        </is>
-      </c>
-      <c r="E54" t="n">
-        <v>24.79</v>
-      </c>
-      <c r="F54" t="n">
-        <v>19.48</v>
-      </c>
-      <c r="G54" t="n">
-        <v>5.309999999999999</v>
-      </c>
-      <c r="H54" t="n">
-        <v>-0.9275000000000011</v>
-      </c>
-      <c r="I54" t="n">
-        <v>1.901977263335279</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>STIM1</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>shTDP-43</t>
-        </is>
-      </c>
-      <c r="C55" t="n">
-        <v>2</v>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>12.06.2026</t>
-        </is>
-      </c>
-      <c r="E55" t="n">
-        <v>25.02</v>
-      </c>
-      <c r="F55" t="n">
-        <v>19.39</v>
-      </c>
-      <c r="G55" t="n">
-        <v>5.629999999999999</v>
-      </c>
-      <c r="H55" t="n">
-        <v>-0.6075000000000008</v>
-      </c>
-      <c r="I55" t="n">
-        <v>1.523616693518236</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>STIM1</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>shTDP-43</t>
-        </is>
-      </c>
-      <c r="C56" t="n">
-        <v>3</v>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>26.06.2026</t>
-        </is>
-      </c>
-      <c r="E56" t="n">
-        <v>24.88</v>
-      </c>
-      <c r="F56" t="n">
-        <v>19.61</v>
-      </c>
-      <c r="G56" t="n">
-        <v>5.27</v>
-      </c>
-      <c r="H56" t="n">
-        <v>-0.9675000000000002</v>
-      </c>
-      <c r="I56" t="n">
-        <v>1.955449122420466</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>STIM1</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>shTDP-43</t>
-        </is>
-      </c>
-      <c r="C57" t="n">
-        <v>4</v>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>10.07.2026</t>
-        </is>
-      </c>
-      <c r="E57" t="n">
-        <v>24.65</v>
-      </c>
-      <c r="F57" t="n">
-        <v>19.52</v>
-      </c>
-      <c r="G57" t="n">
-        <v>5.129999999999999</v>
-      </c>
-      <c r="H57" t="n">
-        <v>-1.107500000000001</v>
-      </c>
-      <c r="I57" t="n">
         <v>2.154719391831541</v>
       </c>
     </row>
@@ -2992,7 +2152,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D57"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3025,7 +2185,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -3043,7 +2203,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -3061,7 +2221,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -3079,7 +2239,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -3169,7 +2329,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -3187,7 +2347,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -3205,7 +2365,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -3223,7 +2383,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -3313,7 +2473,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -3331,7 +2491,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -3349,7 +2509,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -3367,7 +2527,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -3457,7 +2617,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3475,7 +2635,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3493,7 +2653,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3511,7 +2671,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3591,438 +2751,6 @@
       </c>
       <c r="D33" t="n">
         <v>3.089771179918305</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>BCL2</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Control</t>
-        </is>
-      </c>
-      <c r="C34" t="n">
-        <v>1</v>
-      </c>
-      <c r="D34" t="n">
-        <v>0.9913730874626625</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>BCL2</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Control</t>
-        </is>
-      </c>
-      <c r="C35" t="n">
-        <v>2</v>
-      </c>
-      <c r="D35" t="n">
-        <v>1.033472499899175</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>BCL2</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Control</t>
-        </is>
-      </c>
-      <c r="C36" t="n">
-        <v>3</v>
-      </c>
-      <c r="D36" t="n">
-        <v>0.9982686325973916</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>BCL2</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Control</t>
-        </is>
-      </c>
-      <c r="C37" t="n">
-        <v>4</v>
-      </c>
-      <c r="D37" t="n">
-        <v>0.9777245612102334</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>BCL2</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>shTDP-43</t>
-        </is>
-      </c>
-      <c r="C38" t="n">
-        <v>1</v>
-      </c>
-      <c r="D38" t="n">
-        <v>1.941941848684702</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>BCL2</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>shTDP-43</t>
-        </is>
-      </c>
-      <c r="C39" t="n">
-        <v>2</v>
-      </c>
-      <c r="D39" t="n">
-        <v>1.49226111537404</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>BCL2</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>shTDP-43</t>
-        </is>
-      </c>
-      <c r="C40" t="n">
-        <v>3</v>
-      </c>
-      <c r="D40" t="n">
-        <v>1.655767377972946</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>BCL2</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>shTDP-43</t>
-        </is>
-      </c>
-      <c r="C41" t="n">
-        <v>4</v>
-      </c>
-      <c r="D41" t="n">
-        <v>1.824498544489991</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>BAK1</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Control</t>
-        </is>
-      </c>
-      <c r="C42" t="n">
-        <v>1</v>
-      </c>
-      <c r="D42" t="n">
-        <v>1.051537280994008</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>BAK1</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Control</t>
-        </is>
-      </c>
-      <c r="C43" t="n">
-        <v>2</v>
-      </c>
-      <c r="D43" t="n">
-        <v>0.8965773757702972</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>BAK1</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Control</t>
-        </is>
-      </c>
-      <c r="C44" t="n">
-        <v>3</v>
-      </c>
-      <c r="D44" t="n">
-        <v>1.066216194416503</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>BAK1</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Control</t>
-        </is>
-      </c>
-      <c r="C45" t="n">
-        <v>4</v>
-      </c>
-      <c r="D45" t="n">
-        <v>0.9948148855014215</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>BAK1</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>shTDP-43</t>
-        </is>
-      </c>
-      <c r="C46" t="n">
-        <v>1</v>
-      </c>
-      <c r="D46" t="n">
-        <v>0.5008671851173484</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>BAK1</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>shTDP-43</t>
-        </is>
-      </c>
-      <c r="C47" t="n">
-        <v>2</v>
-      </c>
-      <c r="D47" t="n">
-        <v>0.5149484783374492</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>BAK1</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>shTDP-43</t>
-        </is>
-      </c>
-      <c r="C48" t="n">
-        <v>3</v>
-      </c>
-      <c r="D48" t="n">
-        <v>0.4974074427507107</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>BAK1</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>shTDP-43</t>
-        </is>
-      </c>
-      <c r="C49" t="n">
-        <v>4</v>
-      </c>
-      <c r="D49" t="n">
-        <v>0.5043509918951993</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>BAX</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>Control</t>
-        </is>
-      </c>
-      <c r="C50" t="n">
-        <v>1</v>
-      </c>
-      <c r="D50" t="n">
-        <v>0.9090931295275597</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>BAX</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>Control</t>
-        </is>
-      </c>
-      <c r="C51" t="n">
-        <v>2</v>
-      </c>
-      <c r="D51" t="n">
-        <v>1.191269640425871</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>BAX</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>Control</t>
-        </is>
-      </c>
-      <c r="C52" t="n">
-        <v>3</v>
-      </c>
-      <c r="D52" t="n">
-        <v>0.7914115359988518</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>BAX</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>Control</t>
-        </is>
-      </c>
-      <c r="C53" t="n">
-        <v>4</v>
-      </c>
-      <c r="D53" t="n">
-        <v>1.166753665732178</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>BAX</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>shTDP-43</t>
-        </is>
-      </c>
-      <c r="C54" t="n">
-        <v>1</v>
-      </c>
-      <c r="D54" t="n">
-        <v>0.8307578929497527</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>BAX</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>shTDP-43</t>
-        </is>
-      </c>
-      <c r="C55" t="n">
-        <v>2</v>
-      </c>
-      <c r="D55" t="n">
-        <v>0.7435491420613253</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>BAX</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>shTDP-43</t>
-        </is>
-      </c>
-      <c r="C56" t="n">
-        <v>3</v>
-      </c>
-      <c r="D56" t="n">
-        <v>0.9542902250321834</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>BAX</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>shTDP-43</t>
-        </is>
-      </c>
-      <c r="C57" t="n">
-        <v>4</v>
-      </c>
-      <c r="D57" t="n">
-        <v>0.8307578929497527</v>
       </c>
     </row>
   </sheetData>
@@ -4069,7 +2797,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -4087,7 +2815,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -4105,7 +2833,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -4177,7 +2905,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -4195,7 +2923,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -4213,7 +2941,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -4321,7 +3049,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -4339,7 +3067,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -4357,7 +3085,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -4375,7 +3103,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -4465,7 +3193,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -4483,7 +3211,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -4501,7 +3229,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -4519,7 +3247,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -4788,7 +3516,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -4852,7 +3580,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -4916,7 +3644,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -4980,7 +3708,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -5044,7 +3772,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -5108,7 +3836,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -5172,7 +3900,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -5236,7 +3964,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Non-targeting shRNA control</t>
         </is>
       </c>
       <c r="D20" t="n">

</xml_diff>

<commit_message>
Report WST-1 at 48 h only, the time point the thesis reports
Figure 6C, S1, Methods 2.15, Results 3.7, the Figure 6 legend and the Limitations now give the 48 h measurement only. QA: 336 checks.
</commit_message>
<xml_diff>
--- a/supplementary/S1_laboratory_source_data.xlsx
+++ b/supplementary/S1_laboratory_source_data.xlsx
@@ -504,7 +504,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>WST-1 viability, four wells per group, normalised to the mean of the non-targeting (scrambled) shRNA control at the same time point. The experiment was performed three times; these are the four wells of one experiment.</t>
+          <t>WST-1 viability 48 h after seeding, four wells per group, normalised to the mean of the non-targeting (scrambled) shRNA control. The experiment was performed three times; these are the four wells of one experiment.</t>
         </is>
       </c>
     </row>
@@ -3016,7 +3016,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3044,7 +3044,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>24 h</t>
+          <t>48 h</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -3056,13 +3056,13 @@
         <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>97.3063973063973</v>
+        <v>97.47596153846155</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>24 h</t>
+          <t>48 h</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -3074,13 +3074,13 @@
         <v>2</v>
       </c>
       <c r="D3" t="n">
-        <v>103.7037037037037</v>
+        <v>102.6442307692308</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>24 h</t>
+          <t>48 h</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -3092,13 +3092,13 @@
         <v>3</v>
       </c>
       <c r="D4" t="n">
-        <v>97.97979797979798</v>
+        <v>98.4375</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>24 h</t>
+          <t>48 h</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -3110,13 +3110,13 @@
         <v>4</v>
       </c>
       <c r="D5" t="n">
-        <v>101.010101010101</v>
+        <v>101.4423076923077</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>24 h</t>
+          <t>48 h</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -3128,13 +3128,13 @@
         <v>1</v>
       </c>
       <c r="D6" t="n">
-        <v>113.8047138047138</v>
+        <v>59.85576923076923</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>24 h</t>
+          <t>48 h</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -3146,13 +3146,13 @@
         <v>2</v>
       </c>
       <c r="D7" t="n">
-        <v>120.8754208754209</v>
+        <v>63.46153846153847</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>24 h</t>
+          <t>48 h</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -3164,13 +3164,13 @@
         <v>3</v>
       </c>
       <c r="D8" t="n">
-        <v>114.8148148148148</v>
+        <v>60.45673076923077</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>24 h</t>
+          <t>48 h</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -3182,150 +3182,6 @@
         <v>4</v>
       </c>
       <c r="D9" t="n">
-        <v>117.8451178451178</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>48 h</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Non-targeting shRNA control</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>1</v>
-      </c>
-      <c r="D10" t="n">
-        <v>97.47596153846155</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>48 h</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Non-targeting shRNA control</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>2</v>
-      </c>
-      <c r="D11" t="n">
-        <v>102.6442307692308</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>48 h</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Non-targeting shRNA control</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>3</v>
-      </c>
-      <c r="D12" t="n">
-        <v>98.4375</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>48 h</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Non-targeting shRNA control</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>4</v>
-      </c>
-      <c r="D13" t="n">
-        <v>101.4423076923077</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>48 h</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>shTDP-43</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D14" t="n">
-        <v>59.85576923076923</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>48 h</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>shTDP-43</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>2</v>
-      </c>
-      <c r="D15" t="n">
-        <v>63.46153846153847</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>48 h</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>shTDP-43</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>3</v>
-      </c>
-      <c r="D16" t="n">
-        <v>60.45673076923077</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>48 h</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>shTDP-43</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>4</v>
-      </c>
-      <c r="D17" t="n">
         <v>62.3798076923077</v>
       </c>
     </row>
@@ -3340,7 +3196,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3767,7 +3623,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>WST-1 viability 24 h</t>
+          <t>WST-1 viability 48 h</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -3782,7 +3638,7 @@
         <v>100</v>
       </c>
       <c r="F14" t="n">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
@@ -3795,7 +3651,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>WST-1 viability 24 h</t>
+          <t>WST-1 viability 48 h</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -3807,10 +3663,10 @@
         <v>4</v>
       </c>
       <c r="E15" t="n">
-        <v>116.8</v>
+        <v>61.5</v>
       </c>
       <c r="F15" t="n">
-        <v>1.6</v>
+        <v>0.8</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -3819,19 +3675,19 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>0.000243</t>
+          <t>2.14e-07</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>6C</t>
+          <t>6E</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>WST-1 viability 48 h</t>
+          <t>ER Ca2+ release delta F340/F380</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -3840,13 +3696,13 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E16" t="n">
-        <v>100</v>
+        <v>0.268</v>
       </c>
       <c r="F16" t="n">
-        <v>1.2</v>
+        <v>0.042</v>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
@@ -3854,12 +3710,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>6C</t>
+          <t>6E</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>WST-1 viability 48 h</t>
+          <t>ER Ca2+ release delta F340/F380</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -3868,13 +3724,13 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E17" t="n">
-        <v>61.5</v>
+        <v>0.18</v>
       </c>
       <c r="F17" t="n">
-        <v>0.8</v>
+        <v>0.061</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -3883,7 +3739,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2.14e-07</t>
+          <t>0.2989</t>
         </is>
       </c>
     </row>
@@ -3895,7 +3751,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ER Ca2+ release delta F340/F380</t>
+          <t>SOCE delta F340/F380</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -3907,10 +3763,10 @@
         <v>3</v>
       </c>
       <c r="E18" t="n">
-        <v>0.268</v>
+        <v>1.542</v>
       </c>
       <c r="F18" t="n">
-        <v>0.042</v>
+        <v>0.282</v>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
@@ -3923,7 +3779,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ER Ca2+ release delta F340/F380</t>
+          <t>SOCE delta F340/F380</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -3935,10 +3791,10 @@
         <v>3</v>
       </c>
       <c r="E19" t="n">
-        <v>0.18</v>
+        <v>0.245</v>
       </c>
       <c r="F19" t="n">
-        <v>0.061</v>
+        <v>0.083</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -3946,70 +3802,6 @@
         </is>
       </c>
       <c r="H19" t="inlineStr">
-        <is>
-          <t>0.2989</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>6E</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>SOCE delta F340/F380</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Non-targeting shRNA control</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
-        <v>3</v>
-      </c>
-      <c r="E20" t="n">
-        <v>1.542</v>
-      </c>
-      <c r="F20" t="n">
-        <v>0.282</v>
-      </c>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>6E</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>SOCE delta F340/F380</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>shTDP-43</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>3</v>
-      </c>
-      <c r="E21" t="n">
-        <v>0.245</v>
-      </c>
-      <c r="F21" t="n">
-        <v>0.083</v>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>two-tailed Student's t-test</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
         <is>
           <t>0.0115</t>
         </is>

</xml_diff>

<commit_message>
Revert "Report WST-1 at 48 h only, the time point the thesis reports"
This reverts commit b60325d21b4015eb3a92357a296436e859b74180.
</commit_message>
<xml_diff>
--- a/supplementary/S1_laboratory_source_data.xlsx
+++ b/supplementary/S1_laboratory_source_data.xlsx
@@ -504,7 +504,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>WST-1 viability 48 h after seeding, four wells per group, normalised to the mean of the non-targeting (scrambled) shRNA control. The experiment was performed three times; these are the four wells of one experiment.</t>
+          <t>WST-1 viability, four wells per group, normalised to the mean of the non-targeting (scrambled) shRNA control at the same time point. The experiment was performed three times; these are the four wells of one experiment.</t>
         </is>
       </c>
     </row>
@@ -3016,7 +3016,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3044,7 +3044,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>48 h</t>
+          <t>24 h</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -3056,13 +3056,13 @@
         <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>97.47596153846155</v>
+        <v>97.3063973063973</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>48 h</t>
+          <t>24 h</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -3074,13 +3074,13 @@
         <v>2</v>
       </c>
       <c r="D3" t="n">
-        <v>102.6442307692308</v>
+        <v>103.7037037037037</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>48 h</t>
+          <t>24 h</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -3092,13 +3092,13 @@
         <v>3</v>
       </c>
       <c r="D4" t="n">
-        <v>98.4375</v>
+        <v>97.97979797979798</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>48 h</t>
+          <t>24 h</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -3110,13 +3110,13 @@
         <v>4</v>
       </c>
       <c r="D5" t="n">
-        <v>101.4423076923077</v>
+        <v>101.010101010101</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>48 h</t>
+          <t>24 h</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -3128,13 +3128,13 @@
         <v>1</v>
       </c>
       <c r="D6" t="n">
-        <v>59.85576923076923</v>
+        <v>113.8047138047138</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>48 h</t>
+          <t>24 h</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -3146,13 +3146,13 @@
         <v>2</v>
       </c>
       <c r="D7" t="n">
-        <v>63.46153846153847</v>
+        <v>120.8754208754209</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>48 h</t>
+          <t>24 h</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -3164,13 +3164,13 @@
         <v>3</v>
       </c>
       <c r="D8" t="n">
-        <v>60.45673076923077</v>
+        <v>114.8148148148148</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>48 h</t>
+          <t>24 h</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -3182,6 +3182,150 @@
         <v>4</v>
       </c>
       <c r="D9" t="n">
+        <v>117.8451178451178</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>48 h</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Non-targeting shRNA control</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="n">
+        <v>97.47596153846155</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>48 h</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Non-targeting shRNA control</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>2</v>
+      </c>
+      <c r="D11" t="n">
+        <v>102.6442307692308</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>48 h</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Non-targeting shRNA control</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>3</v>
+      </c>
+      <c r="D12" t="n">
+        <v>98.4375</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>48 h</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Non-targeting shRNA control</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>4</v>
+      </c>
+      <c r="D13" t="n">
+        <v>101.4423076923077</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>48 h</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>shTDP-43</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" t="n">
+        <v>59.85576923076923</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>48 h</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>shTDP-43</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" t="n">
+        <v>63.46153846153847</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>48 h</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>shTDP-43</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>3</v>
+      </c>
+      <c r="D16" t="n">
+        <v>60.45673076923077</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>48 h</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>shTDP-43</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>4</v>
+      </c>
+      <c r="D17" t="n">
         <v>62.3798076923077</v>
       </c>
     </row>
@@ -3196,7 +3340,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3623,7 +3767,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>WST-1 viability 48 h</t>
+          <t>WST-1 viability 24 h</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -3638,7 +3782,7 @@
         <v>100</v>
       </c>
       <c r="F14" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
@@ -3651,7 +3795,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>WST-1 viability 48 h</t>
+          <t>WST-1 viability 24 h</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -3663,10 +3807,10 @@
         <v>4</v>
       </c>
       <c r="E15" t="n">
-        <v>61.5</v>
+        <v>116.8</v>
       </c>
       <c r="F15" t="n">
-        <v>0.8</v>
+        <v>1.6</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -3675,19 +3819,19 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2.14e-07</t>
+          <t>0.000243</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>6E</t>
+          <t>6C</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ER Ca2+ release delta F340/F380</t>
+          <t>WST-1 viability 48 h</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -3696,13 +3840,13 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E16" t="n">
-        <v>0.268</v>
+        <v>100</v>
       </c>
       <c r="F16" t="n">
-        <v>0.042</v>
+        <v>1.2</v>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
@@ -3710,12 +3854,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>6E</t>
+          <t>6C</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ER Ca2+ release delta F340/F380</t>
+          <t>WST-1 viability 48 h</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -3724,13 +3868,13 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E17" t="n">
-        <v>0.18</v>
+        <v>61.5</v>
       </c>
       <c r="F17" t="n">
-        <v>0.061</v>
+        <v>0.8</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -3739,7 +3883,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>0.2989</t>
+          <t>2.14e-07</t>
         </is>
       </c>
     </row>
@@ -3751,7 +3895,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>SOCE delta F340/F380</t>
+          <t>ER Ca2+ release delta F340/F380</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -3763,10 +3907,10 @@
         <v>3</v>
       </c>
       <c r="E18" t="n">
-        <v>1.542</v>
+        <v>0.268</v>
       </c>
       <c r="F18" t="n">
-        <v>0.282</v>
+        <v>0.042</v>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
@@ -3779,7 +3923,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>SOCE delta F340/F380</t>
+          <t>ER Ca2+ release delta F340/F380</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -3791,17 +3935,81 @@
         <v>3</v>
       </c>
       <c r="E19" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.061</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>two-tailed Student's t-test</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>0.2989</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>6E</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>SOCE delta F340/F380</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Non-targeting shRNA control</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>3</v>
+      </c>
+      <c r="E20" t="n">
+        <v>1.542</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.282</v>
+      </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>6E</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>SOCE delta F340/F380</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>shTDP-43</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>3</v>
+      </c>
+      <c r="E21" t="n">
         <v>0.245</v>
       </c>
-      <c r="F19" t="n">
+      <c r="F21" t="n">
         <v>0.083</v>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="G21" t="inlineStr">
         <is>
           <t>two-tailed Student's t-test</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="H21" t="inlineStr">
         <is>
           <t>0.0115</t>
         </is>

</xml_diff>

<commit_message>
Add the reviewed manuscript and package corrections; add licences
Reviewed version (MANUSCRIPT_v4_SUBMISSION_REVIEWED.md/.docx), with the original kept
alongside, and the package corrections that go with it:
- S3 lists event coordinates and form lengths for every event class.
- S17 gives 98 samples for GSE138614 and describes run-level group assignment.
- WST-1 is presented descriptively in S1 and Figure 6C.
- README and DATA_AVAILABILITY point to the reviewed manuscript; the consistency check
  runs against it (logs/consistency_check_reviewed.txt, 347 checks).

Licences: MIT for the code (LICENSE); CC BY 4.0 for data, figures, tables and
supplementary files (LICENSE-DATA.md). The manuscript files are not licensed for reuse
before publication.
</commit_message>
<xml_diff>
--- a/supplementary/S1_laboratory_source_data.xlsx
+++ b/supplementary/S1_laboratory_source_data.xlsx
@@ -504,7 +504,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>WST-1 viability, four wells per group, normalised to the mean of the non-targeting (scrambled) shRNA control at the same time point. The experiment was performed three times; these are the four wells of one experiment.</t>
+          <t>WST-1 metabolic signal (not a direct cell count or viability measure), four wells per group, normalised to the mean of the non-targeting (scrambled) shRNA control at the same time point. The experiment was performed three times; these are the four wells of one experiment.</t>
         </is>
       </c>
     </row>
@@ -3037,7 +3037,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>viability_pct_of_control</t>
+          <t>signal_pct_of_control</t>
         </is>
       </c>
     </row>
@@ -3767,7 +3767,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>WST-1 viability 24 h</t>
+          <t>WST-1 signal 24 h</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -3795,7 +3795,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>WST-1 viability 24 h</t>
+          <t>WST-1 signal 24 h</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -3814,14 +3814,10 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>two-tailed Student's t-test</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>0.000243</t>
-        </is>
-      </c>
+          <t>descriptive only; four wells from one experiment</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3831,7 +3827,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>WST-1 viability 48 h</t>
+          <t>WST-1 signal 48 h</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -3859,7 +3855,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>WST-1 viability 48 h</t>
+          <t>WST-1 signal 48 h</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -3878,14 +3874,10 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>two-tailed Student's t-test</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>2.14e-07</t>
-        </is>
-      </c>
+          <t>descriptive only; four wells from one experiment</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">

</xml_diff>

<commit_message>
Finalize four-figure NCI submission package
</commit_message>
<xml_diff>
--- a/supplementary/S1_laboratory_source_data.xlsx
+++ b/supplementary/S1_laboratory_source_data.xlsx
@@ -2,10 +2,6 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TARDBP_qPCR" sheetId="2" state="visible" r:id="rId2"/>
@@ -18,7 +14,6 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thermal_profile" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -28,10 +23,8 @@
   <fonts count="2">
     <font>
       <name val="Calibri"/>
-      <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b val="1"/>
@@ -46,13 +39,7 @@
     </fill>
   </fills>
   <borders count="2">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
+    <border/>
     <border>
       <left style="thin"/>
       <right style="thin"/>
@@ -70,9 +57,8 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -187,72 +173,14 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:ea typeface="Calibri"/>
+        <a:cs typeface="Calibri"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -308,7 +236,7 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="95000"/>
@@ -317,13 +245,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="25400">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="38100">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -357,17 +285,6 @@
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
@@ -422,8 +339,6 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
@@ -480,7 +395,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Relative expression per replicate (2^-ddCt) for the four targets plotted in Figure 6B.</t>
+          <t>Relative expression per replicate (2^-ddCt) for the four targets plotted in Figure 1B.</t>
         </is>
       </c>
     </row>
@@ -492,7 +407,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Fura-2/AM measurements. ER Ca2+ release is the rise in F340/F380 after 10 uM cyclopiazonic acid in Ca2+-free HBS with EGTA; SOCE is the rise after re-addition of 1.5 mM CaCl2. Both as delta(F340/F380) versus the preceding baseline. The three samples of each group come from three independent cultures. The control group is the non-targeting (scrambled) shRNA control.</t>
+          <t>Fura-2/AM data: three measurements per group at 72 h after transduction. The twelve ER-release and SOCE amplitudes agree with the original GraphPad Prism sekil_4.20_fura2.pzfx tables. Figure 2A-B uses unredrawn graphs exported from the original trace project Elmas_130626_Ca2_Trase_Grafikleri.pzf; the original ratio/time tables are supplied separately. Figure 2C-D displays these amplitude measurements and reports two-tailed Student’s t-tests (ER release p = 0.299; Ca²⁺ readdition p = 0.0115). The source Prism graph annotation was corrected to the author-confirmed CPA concentration of 10 µM; trace data and axes were unchanged.</t>
         </is>
       </c>
     </row>
@@ -504,7 +419,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>WST-1 metabolic signal (not a direct cell count or viability measure), four wells per group, normalised to the mean of the non-targeting (scrambled) shRNA control at the same time point. The experiment was performed three times; these are the four wells of one experiment.</t>
+          <t>WST-1 metabolic signal at 48 h, normalised to the non-targeting (scrambled) shRNA control; four wells per group from one available experiment.</t>
         </is>
       </c>
     </row>
@@ -516,7 +431,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Group means, SEM and the statistical test behind every panel of Figure 6.</t>
+          <t>Group means and SEM for Figure 1A-C and Figure 2C-D, with the inferential tests reported in the manuscript. Fura-2 comparisons use two-tailed Student’s t-tests on three measurements per group.</t>
         </is>
       </c>
     </row>
@@ -545,7 +460,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -961,7 +876,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -2142,7 +2057,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -2754,7 +2669,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -3006,7 +2921,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -3016,8 +2931,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3.890000104904175" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="3.559999942779541" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -3044,7 +2965,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>24 h</t>
+          <t>48 h</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -3056,13 +2977,13 @@
         <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>97.3063973063973</v>
+        <v>97.47596153846155</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>24 h</t>
+          <t>48 h</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -3074,13 +2995,13 @@
         <v>2</v>
       </c>
       <c r="D3" t="n">
-        <v>103.7037037037037</v>
+        <v>102.6442307692308</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>24 h</t>
+          <t>48 h</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -3092,13 +3013,13 @@
         <v>3</v>
       </c>
       <c r="D4" t="n">
-        <v>97.97979797979798</v>
+        <v>98.4375</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>24 h</t>
+          <t>48 h</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -3110,13 +3031,13 @@
         <v>4</v>
       </c>
       <c r="D5" t="n">
-        <v>101.010101010101</v>
+        <v>101.4423076923077</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>24 h</t>
+          <t>48 h</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -3128,13 +3049,13 @@
         <v>1</v>
       </c>
       <c r="D6" t="n">
-        <v>113.8047138047138</v>
+        <v>59.85576923076923</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>24 h</t>
+          <t>48 h</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -3146,13 +3067,13 @@
         <v>2</v>
       </c>
       <c r="D7" t="n">
-        <v>120.8754208754209</v>
+        <v>63.46153846153847</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>24 h</t>
+          <t>48 h</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -3164,13 +3085,13 @@
         <v>3</v>
       </c>
       <c r="D8" t="n">
-        <v>114.8148148148148</v>
+        <v>60.45673076923077</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>24 h</t>
+          <t>48 h</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -3182,155 +3103,11 @@
         <v>4</v>
       </c>
       <c r="D9" t="n">
-        <v>117.8451178451178</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>48 h</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Non-targeting shRNA control</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>1</v>
-      </c>
-      <c r="D10" t="n">
-        <v>97.47596153846155</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>48 h</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Non-targeting shRNA control</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>2</v>
-      </c>
-      <c r="D11" t="n">
-        <v>102.6442307692308</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>48 h</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Non-targeting shRNA control</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>3</v>
-      </c>
-      <c r="D12" t="n">
-        <v>98.4375</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>48 h</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Non-targeting shRNA control</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>4</v>
-      </c>
-      <c r="D13" t="n">
-        <v>101.4423076923077</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>48 h</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>shTDP-43</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D14" t="n">
-        <v>59.85576923076923</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>48 h</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>shTDP-43</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>2</v>
-      </c>
-      <c r="D15" t="n">
-        <v>63.46153846153847</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>48 h</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>shTDP-43</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>3</v>
-      </c>
-      <c r="D16" t="n">
-        <v>60.45673076923077</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>48 h</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>shTDP-43</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>4</v>
-      </c>
-      <c r="D17" t="n">
         <v>62.3798076923077</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -3340,8 +3117,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4.78000020980835" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="1.440000057220459" customWidth="1" min="4" max="4"/>
+    <col width="5.440000057220459" customWidth="1" min="5" max="5"/>
+    <col width="5.440000057220459" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
+    <col width="7.329999923706055" customWidth="1" min="8" max="8"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -3388,7 +3175,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>6A</t>
+          <t>1A</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -3410,13 +3197,11 @@
       <c r="F2" t="n">
         <v>0.0242</v>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>6A</t>
+          <t>1A</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -3438,13 +3223,11 @@
       <c r="F3" t="n">
         <v>0.0129</v>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>6A</t>
+          <t>1A</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -3466,13 +3249,11 @@
       <c r="F4" t="n">
         <v>0.0009</v>
       </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>6A</t>
+          <t>1A</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -3491,7 +3272,6 @@
       <c r="E5" t="n">
         <v>94.40000000000001</v>
       </c>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>one-way ANOVA on log2 values, Tukey post hoc</t>
@@ -3506,7 +3286,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>6B</t>
+          <t>1B</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -3528,13 +3308,11 @@
       <c r="F6" t="n">
         <v>0.012</v>
       </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>6B</t>
+          <t>1B</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -3558,19 +3336,17 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>two-tailed Student's t-test</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>0.000303</t>
-        </is>
+          <t>two-tailed Student's t-test; Holm-adjusted across four targets</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>0.000908</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>6B</t>
+          <t>1B</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -3592,13 +3368,11 @@
       <c r="F8" t="n">
         <v>0.015</v>
       </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>6B</t>
+          <t>1B</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -3622,19 +3396,17 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>two-tailed Student's t-test</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>0.000554</t>
-        </is>
+          <t>two-tailed Student's t-test; Holm-adjusted across four targets</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>0.001108</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>6B</t>
+          <t>1B</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -3656,13 +3428,11 @@
       <c r="F10" t="n">
         <v>0.043</v>
       </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>6B</t>
+          <t>1B</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -3686,19 +3456,17 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>two-tailed Student's t-test</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>0.00114</t>
-        </is>
+          <t>two-tailed Student's t-test; Holm-adjusted across four targets</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>0.00114</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>6B</t>
+          <t>1B</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -3720,13 +3488,11 @@
       <c r="F12" t="n">
         <v>0.059</v>
       </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>6B</t>
+          <t>1B</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -3750,24 +3516,22 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>two-tailed Student's t-test</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>9.58e-05</t>
-        </is>
+          <t>two-tailed Student's t-test; Holm-adjusted across four targets</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>0.000383</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>6C</t>
+          <t>1C</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>WST-1 signal 24 h</t>
+          <t>WST-1 signal 48 h</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -3782,20 +3546,18 @@
         <v>100</v>
       </c>
       <c r="F14" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
+        <v>1.2</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>6C</t>
+          <t>1C</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>WST-1 signal 24 h</t>
+          <t>WST-1 signal 48 h</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -3807,27 +3569,26 @@
         <v>4</v>
       </c>
       <c r="E15" t="n">
-        <v>116.8</v>
+        <v>61.5</v>
       </c>
       <c r="F15" t="n">
-        <v>1.6</v>
+        <v>0.8</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>descriptive only; four wells from one experiment</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr"/>
+          <t>Mean ± SEM; one experiment, four wells per group; no inferential test</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>6C</t>
+          <t>2C</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>WST-1 signal 48 h</t>
+          <t>ER Ca2+ release delta F340/F380</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -3836,26 +3597,24 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E16" t="n">
-        <v>100</v>
+        <v>0.268</v>
       </c>
       <c r="F16" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
+        <v>0.042</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>6C</t>
+          <t>2C</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>WST-1 signal 48 h</t>
+          <t>ER Ca2+ release delta F340/F380</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -3864,30 +3623,32 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E17" t="n">
-        <v>61.5</v>
+        <v>0.18</v>
       </c>
       <c r="F17" t="n">
-        <v>0.8</v>
+        <v>0.061</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>descriptive only; four wells from one experiment</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr"/>
+          <t>two-tailed Student's t-test; three measurements per group</t>
+        </is>
+      </c>
+      <c r="H17">
+        <v>0.298923</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>6E</t>
+          <t>2D</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ER Ca2+ release delta F340/F380</t>
+          <t>SOCE delta F340/F380</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -3899,23 +3660,21 @@
         <v>3</v>
       </c>
       <c r="E18" t="n">
-        <v>0.268</v>
+        <v>1.542</v>
       </c>
       <c r="F18" t="n">
-        <v>0.042</v>
-      </c>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
+        <v>0.282</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>6E</t>
+          <t>2D</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ER Ca2+ release delta F340/F380</t>
+          <t>SOCE delta F340/F380</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -3927,88 +3686,22 @@
         <v>3</v>
       </c>
       <c r="E19" t="n">
-        <v>0.18</v>
+        <v>0.245</v>
       </c>
       <c r="F19" t="n">
-        <v>0.061</v>
+        <v>0.083</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>two-tailed Student's t-test</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>0.2989</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>6E</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>SOCE delta F340/F380</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Non-targeting shRNA control</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
-        <v>3</v>
-      </c>
-      <c r="E20" t="n">
-        <v>1.542</v>
-      </c>
-      <c r="F20" t="n">
-        <v>0.282</v>
-      </c>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>6E</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>SOCE delta F340/F380</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>shTDP-43</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>3</v>
-      </c>
-      <c r="E21" t="n">
-        <v>0.245</v>
-      </c>
-      <c r="F21" t="n">
-        <v>0.083</v>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>two-tailed Student's t-test</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>0.0115</t>
-        </is>
+          <t>two-tailed Student's t-test; three measurements per group</t>
+        </is>
+      </c>
+      <c r="H19">
+        <v>0.01153657</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -4222,7 +3915,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -4313,6 +4006,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Polish manuscript layout and simplify sample-size labels
</commit_message>
<xml_diff>
--- a/supplementary/S1_laboratory_source_data.xlsx
+++ b/supplementary/S1_laboratory_source_data.xlsx
@@ -383,7 +383,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Raw Ct values for the four SOCE-associated targets and GAPDH in shTDP-43 cells and the non-targeting (scrambled) shRNA control, four biological replicates per group, same RNA set; experiment window 03.06-10.07.2026.</t>
+          <t>Raw Ct values for the four SOCE-associated targets and GAPDH in shTDP-43 cells and the non-targeting (scrambled) shRNA control, n = 4, same RNA set; experiment window 03.06-10.07.2026.</t>
         </is>
       </c>
     </row>
@@ -407,7 +407,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Fura-2/AM data: three measurements per group at 72 h after transduction. The twelve ER-release and SOCE amplitudes agree with the original GraphPad Prism sekil_4.20_fura2.pzfx tables. Figure 2A-B uses unredrawn graphs exported from the original trace project Elmas_130626_Ca2_Trase_Grafikleri.pzf; the original ratio/time tables are supplied separately. Figure 2C-D displays these amplitude measurements and reports two-tailed Student’s t-tests (ER release p = 0.299; Ca²⁺ readdition p = 0.0115). The source Prism graph annotation was corrected to the author-confirmed CPA concentration of 10 µM; trace data and axes were unchanged.</t>
+          <t>Fura-2/AM data at 72 h after transduction (n = 3). The twelve ER-release and SOCE amplitudes agree with the original GraphPad Prism sekil_4.20_fura2.pzfx tables. Figure 2A-B uses unredrawn graphs exported from the original trace project Elmas_130626_Ca2_Trase_Grafikleri.pzf; the original ratio/time tables are supplied separately. Figure 2C-D displays these amplitude measurements and reports two-tailed Student’s t-tests (ER release p = 0.299; Ca²⁺ readdition p = 0.0115). The source Prism graph annotation was corrected to the author-confirmed CPA concentration of 10 µM; trace data and axes were unchanged.</t>
         </is>
       </c>
     </row>
@@ -419,7 +419,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>WST-1 metabolic signal at 48 h, normalised to the non-targeting (scrambled) shRNA control; four wells per group from one available experiment.</t>
+          <t>WST-1 metabolic signal at 48 h, normalised to the non-targeting (scrambled) shRNA control; n = 4.</t>
         </is>
       </c>
     </row>
@@ -431,7 +431,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Group means and SEM for Figure 1A-C and Figure 2C-D, with the inferential tests reported in the manuscript. Fura-2 comparisons use two-tailed Student’s t-tests on three measurements per group.</t>
+          <t>Group means and SEM for Figure 1A-C and Figure 2C-D, with the inferential tests reported in the manuscript. Fura-2 comparisons use two-tailed Student’s t-tests (n = 3).</t>
         </is>
       </c>
     </row>
@@ -3576,7 +3576,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Mean ± SEM; one experiment, four wells per group; no inferential test</t>
+          <t>Mean ± SEM; n = 4; no inferential test</t>
         </is>
       </c>
     </row>
@@ -3633,10 +3633,10 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>two-tailed Student's t-test; three measurements per group</t>
-        </is>
-      </c>
-      <c r="H17">
+          <t>two-tailed Student's t-test; n = 3</t>
+        </is>
+      </c>
+      <c r="H17" t="n">
         <v>0.298923</v>
       </c>
     </row>
@@ -3693,10 +3693,10 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>two-tailed Student's t-test; three measurements per group</t>
-        </is>
-      </c>
-      <c r="H19">
+          <t>two-tailed Student's t-test; n = 3</t>
+        </is>
+      </c>
+      <c r="H19" t="n">
         <v>0.01153657</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Address manuscript referee review and update source package
</commit_message>
<xml_diff>
--- a/supplementary/S1_laboratory_source_data.xlsx
+++ b/supplementary/S1_laboratory_source_data.xlsx
@@ -2,6 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TARDBP_qPCR" sheetId="2" state="visible" r:id="rId2"/>
@@ -14,6 +18,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thermal_profile" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -23,8 +28,10 @@
   <fonts count="2">
     <font>
       <name val="Calibri"/>
+      <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b val="1"/>
@@ -39,7 +46,13 @@
     </fill>
   </fills>
   <borders count="2">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left style="thin"/>
       <right style="thin"/>
@@ -57,8 +70,9 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -173,14 +187,72 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light"/>
-        <a:ea typeface="Calibri Light"/>
-        <a:cs typeface="Calibri Light"/>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -236,7 +308,7 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="95000"/>
@@ -245,13 +317,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="25400">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -285,6 +357,17 @@
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
@@ -339,6 +422,8 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
@@ -371,7 +456,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>RT-qPCR of TARDBP in three groups, four biological replicates each; raw Ct for TARDBP and GAPDH, dCt, ddCt and 2^-ddCt. Experiment dates 14.04-21.05.2026.</t>
+          <t>RT-qPCR of TARDBP in three groups (n = 4 each); raw Ct for TARDBP and GAPDH, dCt, ddCt and 2^-ddCt. Experiment dates 14.04-21.05.2026.</t>
         </is>
       </c>
     </row>
@@ -407,7 +492,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Fura-2/AM data at 72 h after transduction (n = 3). The twelve ER-release and SOCE amplitudes agree with the original GraphPad Prism sekil_4.20_fura2.pzfx tables. Figure 2A-B uses unredrawn graphs exported from the original trace project Elmas_130626_Ca2_Trase_Grafikleri.pzf; the original ratio/time tables are supplied separately. Figure 2C-D displays these amplitude measurements and reports two-tailed Student’s t-tests (ER release p = 0.299; Ca²⁺ readdition p = 0.0115). The source Prism graph annotation was corrected to the author-confirmed CPA concentration of 10 µM; trace data and axes were unchanged.</t>
+          <t>Fura-2/AM measurements. ER Ca2+ release is the rise in F340/F380 after 10 uM cyclopiazonic acid in Ca2+-free HBS with EGTA; SOCE is the rise after re-addition of nominally 1.5 mM CaCl2. Both are peak delta(F340/F380) versus the preceding baseline (n = 3, descriptive). The control group is the non-targeting (scrambled) shRNA control. The original Prism amplitude table is sekil_4.20_fura2.pzfx. Figure 2A-B uses unredrawn graphs exported from the original trace project Elmas_130626_Ca2_Trase_Grafikleri.pzf; original ratio/time tables are supplied separately. Only the CPA annotation was corrected to the author-confirmed 10 uM; trace data and axes were unchanged.</t>
         </is>
       </c>
     </row>
@@ -419,7 +504,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>WST-1 metabolic signal at 48 h, normalised to the non-targeting (scrambled) shRNA control; n = 4.</t>
+          <t>WST-1 metabolic signal at 48 h (n = 4; not a direct cell count or viability measure), normalised to the mean of the non-targeting (scrambled) shRNA control.</t>
         </is>
       </c>
     </row>
@@ -431,7 +516,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Group means and SEM for Figure 1A-C and Figure 2C-D, with the inferential tests reported in the manuscript. Fura-2 comparisons use two-tailed Student’s t-tests (n = 3).</t>
+          <t>Group means, SEM and the statistical test behind Figures 1 and 2.</t>
         </is>
       </c>
     </row>
@@ -460,7 +545,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -876,7 +961,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -2057,7 +2142,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -2669,7 +2754,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -2921,7 +3006,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -2933,12 +3018,6 @@
   </sheetPr>
   <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="3.890000104904175" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="3.559999942779541" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -3107,7 +3186,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -3119,16 +3198,6 @@
   </sheetPr>
   <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="4.78000020980835" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="1.440000057220459" customWidth="1" min="4" max="4"/>
-    <col width="5.440000057220459" customWidth="1" min="5" max="5"/>
-    <col width="5.440000057220459" customWidth="1" min="6" max="6"/>
-    <col width="42" customWidth="1" min="7" max="7"/>
-    <col width="7.329999923706055" customWidth="1" min="8" max="8"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -3197,6 +3266,8 @@
       <c r="F2" t="n">
         <v>0.0242</v>
       </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3223,6 +3294,8 @@
       <c r="F3" t="n">
         <v>0.0129</v>
       </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3249,6 +3322,8 @@
       <c r="F4" t="n">
         <v>0.0009</v>
       </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3272,6 +3347,7 @@
       <c r="E5" t="n">
         <v>94.40000000000001</v>
       </c>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>one-way ANOVA on log2 values, Tukey post hoc</t>
@@ -3308,6 +3384,8 @@
       <c r="F6" t="n">
         <v>0.012</v>
       </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3339,8 +3417,10 @@
           <t>two-tailed Student's t-test; Holm-adjusted across four targets</t>
         </is>
       </c>
-      <c r="H7" t="n">
-        <v>0.000908</v>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>0.000907664</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -3368,6 +3448,8 @@
       <c r="F8" t="n">
         <v>0.015</v>
       </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3399,8 +3481,10 @@
           <t>two-tailed Student's t-test; Holm-adjusted across four targets</t>
         </is>
       </c>
-      <c r="H9" t="n">
-        <v>0.001108</v>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>0.00110869</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -3428,6 +3512,8 @@
       <c r="F10" t="n">
         <v>0.043</v>
       </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3459,8 +3545,10 @@
           <t>two-tailed Student's t-test; Holm-adjusted across four targets</t>
         </is>
       </c>
-      <c r="H11" t="n">
-        <v>0.00114</v>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>0.00113901</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -3488,6 +3576,8 @@
       <c r="F12" t="n">
         <v>0.059</v>
       </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3519,8 +3609,10 @@
           <t>two-tailed Student's t-test; Holm-adjusted across four targets</t>
         </is>
       </c>
-      <c r="H13" t="n">
-        <v>0.000383</v>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>0.000383066</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -3548,6 +3640,8 @@
       <c r="F14" t="n">
         <v>1.2</v>
       </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3576,9 +3670,10 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Mean ± SEM; n = 4; no inferential test</t>
-        </is>
-      </c>
+          <t>descriptive only; four wells from one experiment</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3605,6 +3700,8 @@
       <c r="F16" t="n">
         <v>0.042</v>
       </c>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3633,12 +3730,10 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>two-tailed Student's t-test; n = 3</t>
-        </is>
-      </c>
-      <c r="H17" t="n">
-        <v>0.298923</v>
-      </c>
+          <t>descriptive; n = 3</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3665,6 +3760,8 @@
       <c r="F18" t="n">
         <v>0.282</v>
       </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3693,15 +3790,13 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>two-tailed Student's t-test; n = 3</t>
-        </is>
-      </c>
-      <c r="H19" t="n">
-        <v>0.01153657</v>
-      </c>
+          <t>descriptive; n = 3</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -3915,7 +4010,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -4006,6 +4101,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Correct experimental units and audit RNA-processing and tissue analyses
</commit_message>
<xml_diff>
--- a/supplementary/S1_laboratory_source_data.xlsx
+++ b/supplementary/S1_laboratory_source_data.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R95e40bd4239747cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TARDBP_qPCR" sheetId="2" r:id="Rb3f2bb48286c4a6d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Target_qPCR_Ct" sheetId="3" r:id="R810899bfcb6646b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Target_qPCR_rel" sheetId="4" r:id="R9da9557cf96a4235"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fura2" sheetId="5" r:id="R5684274583bc4c36"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fura2_per_culture" sheetId="6" r:id="R9c9699f564894882"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WST1" sheetId="7" r:id="R965dd31cc9214072"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary_stats" sheetId="8" r:id="Rc7cb3078d91b48b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Primers" sheetId="9" r:id="Raec4bed26f20458d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thermal_profile" sheetId="10" r:id="R9c2d4384cd5d4b23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rfea85f52ca28460b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TARDBP_qPCR" sheetId="2" r:id="R7c2df2afb1c84419"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Target_qPCR_Ct" sheetId="3" r:id="R4af313dab1a4431f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Target_qPCR_rel" sheetId="4" r:id="R77a197d572a34471"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fura2" sheetId="5" r:id="R73bcd9c3a3764a1a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fura2_per_culture" sheetId="6" r:id="R08939f0ae4a04223"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WST1" sheetId="7" r:id="Rf057bebe82ad41d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary_stats" sheetId="8" r:id="R93b62c8385194994"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Primers" sheetId="9" r:id="R0afadc900880405b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thermal_profile" sheetId="10" r:id="R0947345709e041d1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -52,10 +52,16 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="2">
+  <x:cellXfs count="4">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyAlignment="1">
       <x:alignment horizontal="center" vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -347,6 +353,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="2" max="2" width="100" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="26" hidden="0" customWidth="1"/>
+  </x:cols>
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="1" t="inlineStr">
@@ -360,103 +370,97 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="2">
+    <x:row r="2" ht="65" customHeight="1">
       <x:c r="A2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">TARDBP_qPCR</x:t>
         </x:is>
       </x:c>
-      <x:c r="B2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">RT-qPCR of TARDBP in three groups (n = 4 each); raw Ct for TARDBP and GAPDH, dCt, ddCt and 2^-ddCt. Experiment dates 14.04-21.05.2026.</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="3">
+      <x:c r="B2" s="2" t="str">
+        <x:v>TARDBP RT-qPCR: four technical measurements of the same biological sample per group. Raw Ct, dCt, ddCt and 2^-ddCt are retained. Recorded assay dates do not identify independent cultures.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="65" customHeight="1">
       <x:c r="A3" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Target_qPCR_Ct</x:t>
         </x:is>
       </x:c>
-      <x:c r="B3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Raw Ct values for the four SOCE-associated targets and GAPDH in shTDP-43 cells and the non-targeting (scrambled) shRNA control, n = 4, same RNA set; experiment window 03.06-10.07.2026.</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="4">
+      <x:c r="B3" s="2" t="str">
+        <x:v>Four target genes: raw target and GAPDH Ct values. Four measurements per group are technical repeats of the same biological sample, not independent RNA isolations.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="65" customHeight="1">
       <x:c r="A4" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Target_qPCR_rel</x:t>
         </x:is>
       </x:c>
-      <x:c r="B4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Relative expression per replicate (2^-ddCt) for the four targets plotted in Figure 1B.</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="5">
+      <x:c r="B4" s="2" t="str">
+        <x:v>Relative expression values plotted in Figure 1B. Four technical measurements per target and group; descriptive only.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="180" customHeight="1">
       <x:c r="A5" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Fura2</x:t>
         </x:is>
       </x:c>
-      <x:c r="B5" t="str">
+      <x:c r="B5" s="2" t="str">
         <x:v>Fura-2/AM measurements. ER Ca2+ release is the rise in F340/F380 after 10 uM cyclopiazonic acid in Ca2+-free HBS with EGTA; SOCE is the rise after re-addition of nominally 1.5 mM CaCl2. Both are peak delta(F340/F380) versus the preceding baseline; three wells per group from one culture plate, and well i of both phases is the same recording. This is one biological experiment; the well comparison is descriptive. The control group is the non-targeting (scrambled) shRNA control. The original Prism amplitude table is sekil_4.20_fura2.pzfx. Figure 2A-B uses unredrawn graphs exported from the original trace project Elmas_130626_Ca2_Trase_Grafikleri.pzf; the exported ratio/time tables of these two recordings are in source_data/fura2_traces of the repository and are replotted in Figure 2E. Only the CPA annotation was corrected to the author-confirmed 10 uM; trace data and axes were unchanged.</x:v>
       </x:c>
     </x:row>
-    <x:row r="6">
+    <x:row r="6" ht="65" customHeight="1">
       <x:c r="A6" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Fura2_per_culture</x:t>
         </x:is>
       </x:c>
-      <x:c r="B6" t="str">
+      <x:c r="B6" s="2" t="str">
         <x:v>Both Fura-2 phases per well with the readdition-to-release ratio of that well; one culture plate only. The sheet name is historical.</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
+    <x:row r="7" ht="65" customHeight="1">
       <x:c r="A7" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">WST1</x:t>
         </x:is>
       </x:c>
-      <x:c r="B7" t="inlineStr">
+      <x:c r="B7" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">WST-1 metabolic signal at 48 h (n = 4; not a direct cell count or viability measure), normalised to the mean of the non-targeting (scrambled) shRNA control.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="8">
+    <x:row r="8" ht="65" customHeight="1">
       <x:c r="A8" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Summary_stats</x:t>
         </x:is>
       </x:c>
-      <x:c r="B8" t="str">
-        <x:v>Group means and well-to-well SEM behind Figures 1 and 2; the Fura-2 and WST-1 comparisons are descriptive only.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
+      <x:c r="B8" s="2" t="str">
+        <x:v>Group means and technical-repeat or well-to-well SEM. All laboratory comparisons are descriptive; no inferential p values are reported.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="65" customHeight="1">
       <x:c r="A9" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Primers</x:t>
         </x:is>
       </x:c>
-      <x:c r="B9" t="inlineStr">
+      <x:c r="B9" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Primer sequences, product sizes and annealing temperatures for the RT-qPCR targets and the GAPDH reference.</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="10">
+    <x:row r="10" ht="65" customHeight="1">
       <x:c r="A10" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Thermal_profile</x:t>
         </x:is>
       </x:c>
-      <x:c r="B10" t="inlineStr">
+      <x:c r="B10" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Thermal cycling profile of the RT-qPCR reactions.</x:t>
         </x:is>
@@ -563,10 +567,8 @@
           <x:t xml:space="preserve">group</x:t>
         </x:is>
       </x:c>
-      <x:c r="B1" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">replicate</x:t>
-        </x:is>
+      <x:c r="B1" s="1" t="str">
+        <x:v>technical_repeat</x:v>
       </x:c>
       <x:c r="C1" s="1" t="inlineStr">
         <x:is>
@@ -979,10 +981,8 @@
           <x:t xml:space="preserve">group</x:t>
         </x:is>
       </x:c>
-      <x:c r="C1" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">replicate</x:t>
-        </x:is>
+      <x:c r="C1" s="1" t="str">
+        <x:v>technical_repeat</x:v>
       </x:c>
       <x:c r="D1" s="1" t="inlineStr">
         <x:is>
@@ -2155,10 +2155,8 @@
           <x:t xml:space="preserve">group</x:t>
         </x:is>
       </x:c>
-      <x:c r="C1" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">replicate</x:t>
-        </x:is>
+      <x:c r="C1" s="1" t="str">
+        <x:v>technical_repeat</x:v>
       </x:c>
       <x:c r="D1" s="1" t="inlineStr">
         <x:is>
@@ -3320,6 +3318,16 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="7" max="7" width="58" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="9" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="35" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="35" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="8" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="10" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="10" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
+  </x:cols>
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="1" t="inlineStr">
@@ -3352,7 +3360,7 @@
           <x:t xml:space="preserve">SEM</x:t>
         </x:is>
       </x:c>
-      <x:c r="G1" s="1" t="inlineStr">
+      <x:c r="G1" s="3" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">test</x:t>
         </x:is>
@@ -3363,7 +3371,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="2">
+    <x:row r="2" ht="38" customHeight="1">
       <x:c r="A2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">1A</x:t>
@@ -3388,18 +3396,12 @@
       <x:c r="F2" t="n">
         <x:v>0.0242</x:v>
       </x:c>
-      <x:c r="G2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="H2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="3">
+      <x:c r="G2" s="2" t="str">
+        <x:v>descriptive only; four technical RT-qPCR repeats per group</x:v>
+      </x:c>
+      <x:c r="H2"/>
+    </x:row>
+    <x:row r="3" ht="38" customHeight="1">
       <x:c r="A3" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">1A</x:t>
@@ -3424,18 +3426,12 @@
       <x:c r="F3" t="n">
         <x:v>0.0129</x:v>
       </x:c>
-      <x:c r="G3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="H3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="4">
+      <x:c r="G3" s="2" t="str">
+        <x:v>descriptive only; four technical RT-qPCR repeats per group</x:v>
+      </x:c>
+      <x:c r="H3"/>
+    </x:row>
+    <x:row r="4" ht="38" customHeight="1">
       <x:c r="A4" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">1A</x:t>
@@ -3460,18 +3456,12 @@
       <x:c r="F4" t="n">
         <x:v>0.0009</x:v>
       </x:c>
-      <x:c r="G4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="H4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="5">
+      <x:c r="G4" s="2" t="str">
+        <x:v>descriptive only; four technical RT-qPCR repeats per group</x:v>
+      </x:c>
+      <x:c r="H4"/>
+    </x:row>
+    <x:row r="5" ht="38" customHeight="1">
       <x:c r="A5" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">1A</x:t>
@@ -3498,18 +3488,12 @@
           <x:t xml:space="preserve"/>
         </x:is>
       </x:c>
-      <x:c r="G5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">one-way ANOVA on log2 values, Tukey post hoc</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2.36e-15</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="6">
+      <x:c r="G5" s="2" t="str">
+        <x:v>descriptive only; four technical RT-qPCR repeats per group</x:v>
+      </x:c>
+      <x:c r="H5"/>
+    </x:row>
+    <x:row r="6" ht="38" customHeight="1">
       <x:c r="A6" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">1B</x:t>
@@ -3534,18 +3518,12 @@
       <x:c r="F6" t="n">
         <x:v>0.012</x:v>
       </x:c>
-      <x:c r="G6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="H6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="7">
+      <x:c r="G6" s="2" t="str">
+        <x:v>descriptive only; four technical RT-qPCR repeats per group</x:v>
+      </x:c>
+      <x:c r="H6"/>
+    </x:row>
+    <x:row r="7" ht="38" customHeight="1">
       <x:c r="A7" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">1B</x:t>
@@ -3570,18 +3548,12 @@
       <x:c r="F7" t="n">
         <x:v>0.109</x:v>
       </x:c>
-      <x:c r="G7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">two-tailed Student's t-test; Holm-adjusted across four targets</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">0.000907664</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="8">
+      <x:c r="G7" s="2" t="str">
+        <x:v>descriptive only; four technical RT-qPCR repeats per group</x:v>
+      </x:c>
+      <x:c r="H7"/>
+    </x:row>
+    <x:row r="8" ht="38" customHeight="1">
       <x:c r="A8" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">1B</x:t>
@@ -3606,18 +3578,12 @@
       <x:c r="F8" t="n">
         <x:v>0.015</x:v>
       </x:c>
-      <x:c r="G8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="H8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="9">
+      <x:c r="G8" s="2" t="str">
+        <x:v>descriptive only; four technical RT-qPCR repeats per group</x:v>
+      </x:c>
+      <x:c r="H8"/>
+    </x:row>
+    <x:row r="9" ht="38" customHeight="1">
       <x:c r="A9" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">1B</x:t>
@@ -3642,18 +3608,12 @@
       <x:c r="F9" t="n">
         <x:v>0.132</x:v>
       </x:c>
-      <x:c r="G9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">two-tailed Student's t-test; Holm-adjusted across four targets</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">0.00110869</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="10">
+      <x:c r="G9" s="2" t="str">
+        <x:v>descriptive only; four technical RT-qPCR repeats per group</x:v>
+      </x:c>
+      <x:c r="H9"/>
+    </x:row>
+    <x:row r="10" ht="38" customHeight="1">
       <x:c r="A10" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">1B</x:t>
@@ -3678,18 +3638,12 @@
       <x:c r="F10" t="n">
         <x:v>0.043</x:v>
       </x:c>
-      <x:c r="G10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="H10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="11">
+      <x:c r="G10" s="2" t="str">
+        <x:v>descriptive only; four technical RT-qPCR repeats per group</x:v>
+      </x:c>
+      <x:c r="H10"/>
+    </x:row>
+    <x:row r="11" ht="38" customHeight="1">
       <x:c r="A11" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">1B</x:t>
@@ -3714,18 +3668,12 @@
       <x:c r="F11" t="n">
         <x:v>0.108</x:v>
       </x:c>
-      <x:c r="G11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">two-tailed Student's t-test; Holm-adjusted across four targets</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">0.00113901</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="12">
+      <x:c r="G11" s="2" t="str">
+        <x:v>descriptive only; four technical RT-qPCR repeats per group</x:v>
+      </x:c>
+      <x:c r="H11"/>
+    </x:row>
+    <x:row r="12" ht="38" customHeight="1">
       <x:c r="A12" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">1B</x:t>
@@ -3750,18 +3698,12 @@
       <x:c r="F12" t="n">
         <x:v>0.059</x:v>
       </x:c>
-      <x:c r="G12" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="H12" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="13">
+      <x:c r="G12" s="2" t="str">
+        <x:v>descriptive only; four technical RT-qPCR repeats per group</x:v>
+      </x:c>
+      <x:c r="H12"/>
+    </x:row>
+    <x:row r="13" ht="38" customHeight="1">
       <x:c r="A13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">1B</x:t>
@@ -3786,18 +3728,12 @@
       <x:c r="F13" t="n">
         <x:v>0.233</x:v>
       </x:c>
-      <x:c r="G13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">two-tailed Student's t-test; Holm-adjusted across four targets</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">0.000383066</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="14">
+      <x:c r="G13" s="2" t="str">
+        <x:v>descriptive only; four technical RT-qPCR repeats per group</x:v>
+      </x:c>
+      <x:c r="H13"/>
+    </x:row>
+    <x:row r="14" ht="38" customHeight="1">
       <x:c r="A14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">1C</x:t>
@@ -3822,7 +3758,7 @@
       <x:c r="F14" t="n">
         <x:v>1.2</x:v>
       </x:c>
-      <x:c r="G14" t="inlineStr">
+      <x:c r="G14" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve"/>
         </x:is>
@@ -3833,7 +3769,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="15">
+    <x:row r="15" ht="38" customHeight="1">
       <x:c r="A15" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">1C</x:t>
@@ -3858,7 +3794,7 @@
       <x:c r="F15" t="n">
         <x:v>0.8</x:v>
       </x:c>
-      <x:c r="G15" t="inlineStr">
+      <x:c r="G15" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">descriptive only; four wells from one experiment</x:t>
         </x:is>
@@ -3869,7 +3805,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="16">
+    <x:row r="16" ht="38" customHeight="1">
       <x:c r="A16" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2C</x:t>
@@ -3894,7 +3830,7 @@
       <x:c r="F16" t="n">
         <x:v>0.042</x:v>
       </x:c>
-      <x:c r="G16" t="inlineStr">
+      <x:c r="G16" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve"/>
         </x:is>
@@ -3905,7 +3841,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="17">
+    <x:row r="17" ht="38" customHeight="1">
       <x:c r="A17" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2C</x:t>
@@ -3930,12 +3866,12 @@
       <x:c r="F17" t="n">
         <x:v>0.061</x:v>
       </x:c>
-      <x:c r="G17" t="str">
+      <x:c r="G17" s="2" t="str">
         <x:v>descriptive only; three wells per group on one culture plate</x:v>
       </x:c>
       <x:c r="H17"/>
     </x:row>
-    <x:row r="18">
+    <x:row r="18" ht="38" customHeight="1">
       <x:c r="A18" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2D</x:t>
@@ -3960,7 +3896,7 @@
       <x:c r="F18" t="n">
         <x:v>0.282</x:v>
       </x:c>
-      <x:c r="G18" t="inlineStr">
+      <x:c r="G18" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve"/>
         </x:is>
@@ -3971,7 +3907,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="19">
+    <x:row r="19" ht="38" customHeight="1">
       <x:c r="A19" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2D</x:t>
@@ -3996,12 +3932,12 @@
       <x:c r="F19" t="n">
         <x:v>0.083</x:v>
       </x:c>
-      <x:c r="G19" t="str">
+      <x:c r="G19" s="2" t="str">
         <x:v>descriptive only; three wells per group on one culture plate</x:v>
       </x:c>
       <x:c r="H19"/>
     </x:row>
-    <x:row r="20">
+    <x:row r="20" ht="38" customHeight="1">
       <x:c r="A20" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2C-D</x:t>
@@ -4024,7 +3960,7 @@
       <x:c r="F20" t="n">
         <x:v>1.1</x:v>
       </x:c>
-      <x:c r="G20" t="inlineStr">
+      <x:c r="G20" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve"/>
         </x:is>
@@ -4035,7 +3971,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="21">
+    <x:row r="21" ht="38" customHeight="1">
       <x:c r="A21" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2C-D</x:t>
@@ -4058,7 +3994,7 @@
       <x:c r="F21" t="n">
         <x:v>0.01</x:v>
       </x:c>
-      <x:c r="G21" t="inlineStr">
+      <x:c r="G21" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">descriptive; ratio of the two phases of the same recording</x:t>
         </x:is>

</xml_diff>

<commit_message>
Correct RT-qPCR to four biological replicates and recalculate inference
</commit_message>
<xml_diff>
--- a/supplementary/S1_laboratory_source_data.xlsx
+++ b/supplementary/S1_laboratory_source_data.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rfea85f52ca28460b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TARDBP_qPCR" sheetId="2" r:id="R7c2df2afb1c84419"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Target_qPCR_Ct" sheetId="3" r:id="R4af313dab1a4431f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Target_qPCR_rel" sheetId="4" r:id="R77a197d572a34471"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fura2" sheetId="5" r:id="R73bcd9c3a3764a1a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fura2_per_culture" sheetId="6" r:id="R08939f0ae4a04223"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WST1" sheetId="7" r:id="Rf057bebe82ad41d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary_stats" sheetId="8" r:id="R93b62c8385194994"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Primers" sheetId="9" r:id="R0afadc900880405b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thermal_profile" sheetId="10" r:id="R0947345709e041d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R1bf261c67abb4b78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TARDBP_qPCR" sheetId="2" r:id="Ra48d13d160534528"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Target_qPCR_Ct" sheetId="3" r:id="Rec2fdaf19d7c45c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Target_qPCR_rel" sheetId="4" r:id="Rb70280b497054470"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fura2" sheetId="5" r:id="R664a73f6298544a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fura2_per_culture" sheetId="6" r:id="R3308f63c9e284bb1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WST1" sheetId="7" r:id="R712e6cbd67fd4ac4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary_stats" sheetId="8" r:id="Rf4f8e8792d7f4b75"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Primers" sheetId="9" r:id="R06f1f02d1e634ca1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thermal_profile" sheetId="10" r:id="R205bdf77d7d54127"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -22,6 +22,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:numFmts count="1">
+    <x:numFmt numFmtId="200" formatCode="0.00E+00"/>
+  </x:numFmts>
   <x:fonts count="2">
     <x:font>
       <x:sz val="11"/>
@@ -52,7 +55,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="4">
+  <x:cellXfs count="5">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyAlignment="1">
       <x:alignment horizontal="center" vertical="top"/>
@@ -63,6 +66,7 @@
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -377,7 +381,7 @@
         </x:is>
       </x:c>
       <x:c r="B2" s="2" t="str">
-        <x:v>TARDBP RT-qPCR: four technical measurements of the same biological sample per group. Raw Ct, dCt, ddCt and 2^-ddCt are retained. Recorded assay dates do not identify independent cultures.</x:v>
+        <x:v>TARDBP RT-qPCR: four biological replicates per group. Raw Ct, dCt, ddCt and 2^-ddCt are retained.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="65" customHeight="1">
@@ -387,7 +391,7 @@
         </x:is>
       </x:c>
       <x:c r="B3" s="2" t="str">
-        <x:v>Four target genes: raw target and GAPDH Ct values. Four measurements per group are technical repeats of the same biological sample, not independent RNA isolations.</x:v>
+        <x:v>Four target genes: raw target and GAPDH Ct values from four biological replicates per group. The target-gene assays share an RNA set; TARDBP uses a separate set.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="65" customHeight="1">
@@ -397,7 +401,7 @@
         </x:is>
       </x:c>
       <x:c r="B4" s="2" t="str">
-        <x:v>Relative expression values plotted in Figure 1B. Four technical measurements per target and group; descriptive only.</x:v>
+        <x:v>Relative expression values plotted in Figure 1B. Four biological replicates per target and group.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="180" customHeight="1">
@@ -439,7 +443,7 @@
         </x:is>
       </x:c>
       <x:c r="B8" s="2" t="str">
-        <x:v>Group means and technical-repeat or well-to-well SEM. All laboratory comparisons are descriptive; no inferential p values are reported.</x:v>
+        <x:v>Group means and SEM across biological replicates for RT-qPCR. Two-sided Welch tests on dCt; Holm correction across four targets and separately across two TARDBP contrasts. Fura-2 and WST-1 summaries describe well-to-well variation only.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="65" customHeight="1">
@@ -560,6 +564,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
+  </x:cols>
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="1" t="inlineStr">
@@ -568,7 +575,7 @@
         </x:is>
       </x:c>
       <x:c r="B1" s="1" t="str">
-        <x:v>technical_repeat</x:v>
+        <x:v>biological_replicate</x:v>
       </x:c>
       <x:c r="C1" s="1" t="inlineStr">
         <x:is>
@@ -969,6 +976,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
+  </x:cols>
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="1" t="inlineStr">
@@ -982,7 +992,7 @@
         </x:is>
       </x:c>
       <x:c r="C1" s="1" t="str">
-        <x:v>technical_repeat</x:v>
+        <x:v>biological_replicate</x:v>
       </x:c>
       <x:c r="D1" s="1" t="inlineStr">
         <x:is>
@@ -2143,6 +2153,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
+  </x:cols>
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="1" t="inlineStr">
@@ -2156,7 +2169,7 @@
         </x:is>
       </x:c>
       <x:c r="C1" s="1" t="str">
-        <x:v>technical_repeat</x:v>
+        <x:v>biological_replicate</x:v>
       </x:c>
       <x:c r="D1" s="1" t="inlineStr">
         <x:is>
@@ -3397,9 +3410,9 @@
         <x:v>0.0242</x:v>
       </x:c>
       <x:c r="G2" s="2" t="str">
-        <x:v>descriptive only; four technical RT-qPCR repeats per group</x:v>
-      </x:c>
-      <x:c r="H2"/>
+        <x:v>four biological replicates per group; mean and SEM</x:v>
+      </x:c>
+      <x:c r="H2" s="4"/>
     </x:row>
     <x:row r="3" ht="38" customHeight="1">
       <x:c r="A3" t="inlineStr">
@@ -3427,9 +3440,9 @@
         <x:v>0.0129</x:v>
       </x:c>
       <x:c r="G3" s="2" t="str">
-        <x:v>descriptive only; four technical RT-qPCR repeats per group</x:v>
-      </x:c>
-      <x:c r="H3"/>
+        <x:v>four biological replicates per group; mean and SEM</x:v>
+      </x:c>
+      <x:c r="H3" s="4"/>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
       <x:c r="A4" t="inlineStr">
@@ -3457,9 +3470,9 @@
         <x:v>0.0009</x:v>
       </x:c>
       <x:c r="G4" s="2" t="str">
-        <x:v>descriptive only; four technical RT-qPCR repeats per group</x:v>
-      </x:c>
-      <x:c r="H4"/>
+        <x:v>four biological replicates per group; mean and SEM</x:v>
+      </x:c>
+      <x:c r="H4" s="4"/>
     </x:row>
     <x:row r="5" ht="38" customHeight="1">
       <x:c r="A5" t="inlineStr">
@@ -3489,9 +3502,11 @@
         </x:is>
       </x:c>
       <x:c r="G5" s="2" t="str">
-        <x:v>descriptive only; four technical RT-qPCR repeats per group</x:v>
-      </x:c>
-      <x:c r="H5"/>
+        <x:v>Welch dCt; max Holm-adjusted p of two TARDBP contrasts</x:v>
+      </x:c>
+      <x:c r="H5" s="4" t="n">
+        <x:v>3.1995558426905583e-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="38" customHeight="1">
       <x:c r="A6" t="inlineStr">
@@ -3519,9 +3534,9 @@
         <x:v>0.012</x:v>
       </x:c>
       <x:c r="G6" s="2" t="str">
-        <x:v>descriptive only; four technical RT-qPCR repeats per group</x:v>
-      </x:c>
-      <x:c r="H6"/>
+        <x:v>four biological replicates per group; mean and SEM</x:v>
+      </x:c>
+      <x:c r="H6" s="4"/>
     </x:row>
     <x:row r="7" ht="38" customHeight="1">
       <x:c r="A7" t="inlineStr">
@@ -3549,9 +3564,11 @@
         <x:v>0.109</x:v>
       </x:c>
       <x:c r="G7" s="2" t="str">
-        <x:v>descriptive only; four technical RT-qPCR repeats per group</x:v>
-      </x:c>
-      <x:c r="H7"/>
+        <x:v>two-sided Welch dCt; Holm-adjusted across four targets</x:v>
+      </x:c>
+      <x:c r="H7" s="4" t="n">
+        <x:v>0.003961679552801206</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="38" customHeight="1">
       <x:c r="A8" t="inlineStr">
@@ -3579,9 +3596,9 @@
         <x:v>0.015</x:v>
       </x:c>
       <x:c r="G8" s="2" t="str">
-        <x:v>descriptive only; four technical RT-qPCR repeats per group</x:v>
-      </x:c>
-      <x:c r="H8"/>
+        <x:v>four biological replicates per group; mean and SEM</x:v>
+      </x:c>
+      <x:c r="H8" s="4"/>
     </x:row>
     <x:row r="9" ht="38" customHeight="1">
       <x:c r="A9" t="inlineStr">
@@ -3609,9 +3626,11 @@
         <x:v>0.132</x:v>
       </x:c>
       <x:c r="G9" s="2" t="str">
-        <x:v>descriptive only; four technical RT-qPCR repeats per group</x:v>
-      </x:c>
-      <x:c r="H9"/>
+        <x:v>two-sided Welch dCt; Holm-adjusted across four targets</x:v>
+      </x:c>
+      <x:c r="H9" s="4" t="n">
+        <x:v>0.003961679552801206</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="38" customHeight="1">
       <x:c r="A10" t="inlineStr">
@@ -3639,9 +3658,9 @@
         <x:v>0.043</x:v>
       </x:c>
       <x:c r="G10" s="2" t="str">
-        <x:v>descriptive only; four technical RT-qPCR repeats per group</x:v>
-      </x:c>
-      <x:c r="H10"/>
+        <x:v>four biological replicates per group; mean and SEM</x:v>
+      </x:c>
+      <x:c r="H10" s="4"/>
     </x:row>
     <x:row r="11" ht="38" customHeight="1">
       <x:c r="A11" t="inlineStr">
@@ -3669,9 +3688,11 @@
         <x:v>0.108</x:v>
       </x:c>
       <x:c r="G11" s="2" t="str">
-        <x:v>descriptive only; four technical RT-qPCR repeats per group</x:v>
-      </x:c>
-      <x:c r="H11"/>
+        <x:v>two-sided Welch dCt; Holm-adjusted across four targets</x:v>
+      </x:c>
+      <x:c r="H11" s="4" t="n">
+        <x:v>0.0026092887594562526</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="38" customHeight="1">
       <x:c r="A12" t="inlineStr">
@@ -3699,9 +3720,9 @@
         <x:v>0.059</x:v>
       </x:c>
       <x:c r="G12" s="2" t="str">
-        <x:v>descriptive only; four technical RT-qPCR repeats per group</x:v>
-      </x:c>
-      <x:c r="H12"/>
+        <x:v>four biological replicates per group; mean and SEM</x:v>
+      </x:c>
+      <x:c r="H12" s="4"/>
     </x:row>
     <x:row r="13" ht="38" customHeight="1">
       <x:c r="A13" t="inlineStr">
@@ -3729,9 +3750,11 @@
         <x:v>0.233</x:v>
       </x:c>
       <x:c r="G13" s="2" t="str">
-        <x:v>descriptive only; four technical RT-qPCR repeats per group</x:v>
-      </x:c>
-      <x:c r="H13"/>
+        <x:v>two-sided Welch dCt; Holm-adjusted across four targets</x:v>
+      </x:c>
+      <x:c r="H13" s="4" t="n">
+        <x:v>0.0000676605356856677</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="38" customHeight="1">
       <x:c r="A14" t="inlineStr">

</xml_diff>